<commit_message>
vault backup: 2026-08-10 19:13:02
</commit_message>
<xml_diff>
--- a/ContabilidadeFinanceira/Treinos/Ex1_GraoDeOuro.xlsx
+++ b/ContabilidadeFinanceira/Treinos/Ex1_GraoDeOuro.xlsx
@@ -44,14 +44,14 @@
       <b val="1"/>
     </font>
     <font>
+      <i val="1"/>
+      <color rgb="00808080"/>
+      <sz val="8"/>
+    </font>
+    <font>
       <b val="1"/>
       <i val="1"/>
       <sz val="9"/>
-    </font>
-    <font>
-      <i val="1"/>
-      <color rgb="00808080"/>
-      <sz val="8"/>
     </font>
     <font>
       <b val="1"/>
@@ -120,28 +120,30 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -522,17 +524,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H16"/>
+  <dimension ref="A1:K17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="11" customWidth="1" min="1" max="1"/>
-    <col width="52" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="4" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
-    <col width="4" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="46" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="3" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="3" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="8" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -545,14 +550,14 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Uma linha por movimento. Se a transação mexe em duas contas do mesmo lado (ex: sai caixa, entra estoque), usa as duas linhas.</t>
+          <t>Uma linha por movimento: escreve a conta e o valor, com sinal. Transação que mexe em três contas do mesmo lado usa as três linhas. A coluna Check acusa se aquela transação fechou.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Transação</t>
+          <t>Nº</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -565,305 +570,390 @@
           <t>ATIVO</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="4" t="n"/>
+      <c r="E4" s="3" t="inlineStr">
         <is>
           <t>=</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="F4" s="3" t="inlineStr">
         <is>
           <t>PASSIVO</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="G4" s="4" t="n"/>
+      <c r="H4" s="3" t="inlineStr">
         <is>
           <t>+</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="I4" s="3" t="inlineStr">
         <is>
           <t>PATRIMÔNIO LÍQUIDO</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr">
+      <c r="J4" s="4" t="n"/>
+      <c r="K4" s="3" t="inlineStr">
         <is>
           <t>Check</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="15" customHeight="1">
-      <c r="A5" s="4" t="n">
+    <row r="5">
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>conta</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>valor</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>conta</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>valor</t>
+        </is>
+      </c>
+      <c r="I5" s="5" t="inlineStr">
+        <is>
+          <t>conta</t>
+        </is>
+      </c>
+      <c r="J5" s="5" t="inlineStr">
+        <is>
+          <t>valor</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="B5" s="5" t="inlineStr">
+      <c r="B6" s="7" t="inlineStr">
         <is>
           <t>Integralização de capital de R$ 80.000 em dinheiro</t>
         </is>
       </c>
-      <c r="C5" s="6" t="n"/>
-      <c r="D5" s="7" t="inlineStr">
+      <c r="C6" s="8" t="n"/>
+      <c r="D6" s="9" t="n"/>
+      <c r="E6" s="10" t="inlineStr">
         <is>
           <t>=</t>
         </is>
       </c>
-      <c r="E5" s="6" t="n"/>
-      <c r="F5" s="7" t="inlineStr">
+      <c r="F6" s="8" t="n"/>
+      <c r="G6" s="9" t="n"/>
+      <c r="H6" s="10" t="inlineStr">
         <is>
           <t>+</t>
         </is>
       </c>
-      <c r="G5" s="6" t="n"/>
-      <c r="H5" s="8">
-        <f>IF(COUNT(C5:C6,E5:E6,G5:G6)=0,"",IF(SUM(C5:C6)-SUM(E5:E6)-SUM(G5:G6)=0,"✔","✗"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="6">
-      <c r="C6" s="6" t="n"/>
-      <c r="D6" s="7" t="inlineStr">
+      <c r="I6" s="8" t="n"/>
+      <c r="J6" s="9" t="n"/>
+      <c r="K6" s="6">
+        <f>IF(COUNT(D6:D7,G6:G7,J6:J7)=0,"",IF(SUM(D6:D7)-SUM(G6:G7)-SUM(J6:J7)=0,"✔","✗"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="C7" s="8" t="n"/>
+      <c r="D7" s="9" t="n"/>
+      <c r="E7" s="10" t="inlineStr">
         <is>
           <t>=</t>
         </is>
       </c>
-      <c r="E6" s="6" t="n"/>
-      <c r="F6" s="7" t="inlineStr">
+      <c r="F7" s="8" t="n"/>
+      <c r="G7" s="9" t="n"/>
+      <c r="H7" s="10" t="inlineStr">
         <is>
           <t>+</t>
         </is>
       </c>
-      <c r="G6" s="6" t="n"/>
-    </row>
-    <row r="7" ht="15" customHeight="1">
-      <c r="A7" s="4" t="n">
+      <c r="I7" s="8" t="n"/>
+      <c r="J7" s="9" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="B7" s="5" t="inlineStr">
+      <c r="B8" s="7" t="inlineStr">
         <is>
           <t>Compra à vista de máquina de espresso e mobiliário por R$ 30.000</t>
         </is>
       </c>
-      <c r="C7" s="6" t="n"/>
-      <c r="D7" s="7" t="inlineStr">
+      <c r="C8" s="8" t="n"/>
+      <c r="D8" s="9" t="n"/>
+      <c r="E8" s="10" t="inlineStr">
         <is>
           <t>=</t>
         </is>
       </c>
-      <c r="E7" s="6" t="n"/>
-      <c r="F7" s="7" t="inlineStr">
+      <c r="F8" s="8" t="n"/>
+      <c r="G8" s="9" t="n"/>
+      <c r="H8" s="10" t="inlineStr">
         <is>
           <t>+</t>
         </is>
       </c>
-      <c r="G7" s="6" t="n"/>
-      <c r="H7" s="8">
-        <f>IF(COUNT(C7:C8,E7:E8,G7:G8)=0,"",IF(SUM(C7:C8)-SUM(E7:E8)-SUM(G7:G8)=0,"✔","✗"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="8">
-      <c r="C8" s="6" t="n"/>
-      <c r="D8" s="7" t="inlineStr">
+      <c r="I8" s="8" t="n"/>
+      <c r="J8" s="9" t="n"/>
+      <c r="K8" s="6">
+        <f>IF(COUNT(D8:D9,G8:G9,J8:J9)=0,"",IF(SUM(D8:D9)-SUM(G8:G9)-SUM(J8:J9)=0,"✔","✗"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="C9" s="8" t="n"/>
+      <c r="D9" s="9" t="n"/>
+      <c r="E9" s="10" t="inlineStr">
         <is>
           <t>=</t>
         </is>
       </c>
-      <c r="E8" s="6" t="n"/>
-      <c r="F8" s="7" t="inlineStr">
+      <c r="F9" s="8" t="n"/>
+      <c r="G9" s="9" t="n"/>
+      <c r="H9" s="10" t="inlineStr">
         <is>
           <t>+</t>
         </is>
       </c>
-      <c r="G8" s="6" t="n"/>
-    </row>
-    <row r="9" ht="15" customHeight="1">
-      <c r="A9" s="4" t="n">
+      <c r="I9" s="8" t="n"/>
+      <c r="J9" s="9" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="B9" s="5" t="inlineStr">
+      <c r="B10" s="7" t="inlineStr">
         <is>
           <t>Compra de café e insumos por R$ 24.000, metade à vista e metade a prazo</t>
         </is>
       </c>
-      <c r="C9" s="6" t="n"/>
-      <c r="D9" s="7" t="inlineStr">
+      <c r="C10" s="8" t="n"/>
+      <c r="D10" s="9" t="n"/>
+      <c r="E10" s="10" t="inlineStr">
         <is>
           <t>=</t>
         </is>
       </c>
-      <c r="E9" s="6" t="n"/>
-      <c r="F9" s="7" t="inlineStr">
+      <c r="F10" s="8" t="n"/>
+      <c r="G10" s="9" t="n"/>
+      <c r="H10" s="10" t="inlineStr">
         <is>
           <t>+</t>
         </is>
       </c>
-      <c r="G9" s="6" t="n"/>
-      <c r="H9" s="8">
-        <f>IF(COUNT(C9:C10,E9:E10,G9:G10)=0,"",IF(SUM(C9:C10)-SUM(E9:E10)-SUM(G9:G10)=0,"✔","✗"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="10">
-      <c r="C10" s="6" t="n"/>
-      <c r="D10" s="7" t="inlineStr">
+      <c r="I10" s="8" t="n"/>
+      <c r="J10" s="9" t="n"/>
+      <c r="K10" s="6">
+        <f>IF(COUNT(D10:D11,G10:G11,J10:J11)=0,"",IF(SUM(D10:D11)-SUM(G10:G11)-SUM(J10:J11)=0,"✔","✗"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="C11" s="8" t="n"/>
+      <c r="D11" s="9" t="n"/>
+      <c r="E11" s="10" t="inlineStr">
         <is>
           <t>=</t>
         </is>
       </c>
-      <c r="E10" s="6" t="n"/>
-      <c r="F10" s="7" t="inlineStr">
+      <c r="F11" s="8" t="n"/>
+      <c r="G11" s="9" t="n"/>
+      <c r="H11" s="10" t="inlineStr">
         <is>
           <t>+</t>
         </is>
       </c>
-      <c r="G10" s="6" t="n"/>
-    </row>
-    <row r="11" ht="15" customHeight="1">
-      <c r="A11" s="4" t="n">
+      <c r="I11" s="8" t="n"/>
+      <c r="J11" s="9" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="B11" s="5" t="inlineStr">
+      <c r="B12" s="7" t="inlineStr">
         <is>
           <t>Venda de metade do estoque por R$ 27.000 à vista (custo de R$ 12.000)</t>
         </is>
       </c>
-      <c r="C11" s="6" t="n"/>
-      <c r="D11" s="7" t="inlineStr">
+      <c r="C12" s="8" t="n"/>
+      <c r="D12" s="9" t="n"/>
+      <c r="E12" s="10" t="inlineStr">
         <is>
           <t>=</t>
         </is>
       </c>
-      <c r="E11" s="6" t="n"/>
-      <c r="F11" s="7" t="inlineStr">
+      <c r="F12" s="8" t="n"/>
+      <c r="G12" s="9" t="n"/>
+      <c r="H12" s="10" t="inlineStr">
         <is>
           <t>+</t>
         </is>
       </c>
-      <c r="G11" s="6" t="n"/>
-      <c r="H11" s="8">
-        <f>IF(COUNT(C11:C12,E11:E12,G11:G12)=0,"",IF(SUM(C11:C12)-SUM(E11:E12)-SUM(G11:G12)=0,"✔","✗"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="12">
-      <c r="C12" s="6" t="n"/>
-      <c r="D12" s="7" t="inlineStr">
+      <c r="I12" s="8" t="n"/>
+      <c r="J12" s="9" t="n"/>
+      <c r="K12" s="6">
+        <f>IF(COUNT(D12:D13,G12:G13,J12:J13)=0,"",IF(SUM(D12:D13)-SUM(G12:G13)-SUM(J12:J13)=0,"✔","✗"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="C13" s="8" t="n"/>
+      <c r="D13" s="9" t="n"/>
+      <c r="E13" s="10" t="inlineStr">
         <is>
           <t>=</t>
         </is>
       </c>
-      <c r="E12" s="6" t="n"/>
-      <c r="F12" s="7" t="inlineStr">
+      <c r="F13" s="8" t="n"/>
+      <c r="G13" s="9" t="n"/>
+      <c r="H13" s="10" t="inlineStr">
         <is>
           <t>+</t>
         </is>
       </c>
-      <c r="G12" s="6" t="n"/>
-    </row>
-    <row r="13" ht="15" customHeight="1">
-      <c r="A13" s="4" t="n">
+      <c r="I13" s="8" t="n"/>
+      <c r="J13" s="9" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="B13" s="5" t="inlineStr">
+      <c r="B14" s="7" t="inlineStr">
         <is>
           <t>Pagamento de salários e aluguel do mês, R$ 6.000 à vista</t>
         </is>
       </c>
-      <c r="C13" s="6" t="n"/>
-      <c r="D13" s="7" t="inlineStr">
+      <c r="C14" s="8" t="n"/>
+      <c r="D14" s="9" t="n"/>
+      <c r="E14" s="10" t="inlineStr">
         <is>
           <t>=</t>
         </is>
       </c>
-      <c r="E13" s="6" t="n"/>
-      <c r="F13" s="7" t="inlineStr">
+      <c r="F14" s="8" t="n"/>
+      <c r="G14" s="9" t="n"/>
+      <c r="H14" s="10" t="inlineStr">
         <is>
           <t>+</t>
         </is>
       </c>
-      <c r="G13" s="6" t="n"/>
-      <c r="H13" s="8">
-        <f>IF(COUNT(C13:C14,E13:E14,G13:G14)=0,"",IF(SUM(C13:C14)-SUM(E13:E14)-SUM(G13:G14)=0,"✔","✗"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="14">
-      <c r="C14" s="6" t="n"/>
-      <c r="D14" s="7" t="inlineStr">
+      <c r="I14" s="8" t="n"/>
+      <c r="J14" s="9" t="n"/>
+      <c r="K14" s="6">
+        <f>IF(COUNT(D14:D15,G14:G15,J14:J15)=0,"",IF(SUM(D14:D15)-SUM(G14:G15)-SUM(J14:J15)=0,"✔","✗"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="C15" s="8" t="n"/>
+      <c r="D15" s="9" t="n"/>
+      <c r="E15" s="10" t="inlineStr">
         <is>
           <t>=</t>
         </is>
       </c>
-      <c r="E14" s="6" t="n"/>
-      <c r="F14" s="7" t="inlineStr">
+      <c r="F15" s="8" t="n"/>
+      <c r="G15" s="9" t="n"/>
+      <c r="H15" s="10" t="inlineStr">
         <is>
           <t>+</t>
         </is>
       </c>
-      <c r="G14" s="6" t="n"/>
-    </row>
-    <row r="15" ht="15" customHeight="1">
-      <c r="A15" s="4" t="n">
+      <c r="I15" s="8" t="n"/>
+      <c r="J15" s="9" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="B15" s="5" t="inlineStr">
+      <c r="B16" s="7" t="inlineStr">
         <is>
           <t>Pagamento de metade do que devia aos fornecedores</t>
         </is>
       </c>
-      <c r="C15" s="6" t="n"/>
-      <c r="D15" s="7" t="inlineStr">
+      <c r="C16" s="8" t="n"/>
+      <c r="D16" s="9" t="n"/>
+      <c r="E16" s="10" t="inlineStr">
         <is>
           <t>=</t>
         </is>
       </c>
-      <c r="E15" s="6" t="n"/>
-      <c r="F15" s="7" t="inlineStr">
+      <c r="F16" s="8" t="n"/>
+      <c r="G16" s="9" t="n"/>
+      <c r="H16" s="10" t="inlineStr">
         <is>
           <t>+</t>
         </is>
       </c>
-      <c r="G15" s="6" t="n"/>
-      <c r="H15" s="8">
-        <f>IF(COUNT(C15:C16,E15:E16,G15:G16)=0,"",IF(SUM(C15:C16)-SUM(E15:E16)-SUM(G15:G16)=0,"✔","✗"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="16">
-      <c r="C16" s="6" t="n"/>
-      <c r="D16" s="7" t="inlineStr">
+      <c r="I16" s="8" t="n"/>
+      <c r="J16" s="9" t="n"/>
+      <c r="K16" s="6">
+        <f>IF(COUNT(D16:D17,G16:G17,J16:J17)=0,"",IF(SUM(D16:D17)-SUM(G16:G17)-SUM(J16:J17)=0,"✔","✗"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="C17" s="8" t="n"/>
+      <c r="D17" s="9" t="n"/>
+      <c r="E17" s="10" t="inlineStr">
         <is>
           <t>=</t>
         </is>
       </c>
-      <c r="E16" s="6" t="n"/>
-      <c r="F16" s="7" t="inlineStr">
+      <c r="F17" s="8" t="n"/>
+      <c r="G17" s="9" t="n"/>
+      <c r="H17" s="10" t="inlineStr">
         <is>
           <t>+</t>
         </is>
       </c>
-      <c r="G16" s="6" t="n"/>
+      <c r="I17" s="8" t="n"/>
+      <c r="J17" s="9" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="18">
-    <mergeCell ref="A5:A6"/>
-    <mergeCell ref="B9:B10"/>
-    <mergeCell ref="H5:H6"/>
-    <mergeCell ref="H13:H14"/>
-    <mergeCell ref="H9:H10"/>
-    <mergeCell ref="A9:A10"/>
-    <mergeCell ref="A13:A14"/>
-    <mergeCell ref="B13:B14"/>
-    <mergeCell ref="A15:A16"/>
-    <mergeCell ref="A7:A8"/>
-    <mergeCell ref="B7:B8"/>
-    <mergeCell ref="B11:B12"/>
-    <mergeCell ref="H7:H8"/>
-    <mergeCell ref="H15:H16"/>
-    <mergeCell ref="H11:H12"/>
-    <mergeCell ref="B5:B6"/>
-    <mergeCell ref="A11:A12"/>
-    <mergeCell ref="B15:B16"/>
+  <mergeCells count="21">
+    <mergeCell ref="F4:G4"/>
+    <mergeCell ref="B12:B13"/>
+    <mergeCell ref="B8:B9"/>
+    <mergeCell ref="A16:A17"/>
+    <mergeCell ref="A6:A7"/>
+    <mergeCell ref="B14:B15"/>
+    <mergeCell ref="C4:D4"/>
+    <mergeCell ref="A12:A13"/>
+    <mergeCell ref="K12:K13"/>
+    <mergeCell ref="B10:B11"/>
+    <mergeCell ref="B6:B7"/>
+    <mergeCell ref="A14:A15"/>
+    <mergeCell ref="A8:A9"/>
+    <mergeCell ref="K14:K15"/>
+    <mergeCell ref="K8:K9"/>
+    <mergeCell ref="A10:A11"/>
+    <mergeCell ref="K10:K11"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="K16:K17"/>
+    <mergeCell ref="K6:K7"/>
+    <mergeCell ref="B16:B17"/>
   </mergeCells>
+  <dataValidations count="3">
+    <dataValidation sqref="C6 C7 C8 C9 C10 C11 C12 C13 C14 C15 C16 C17" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Caixa,Estoque,Imobilizado"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F6 F7 F8 F9 F10 F11 F12 F13 F14 F15 F16 F17" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Contas a Pagar"</formula1>
+    </dataValidation>
+    <dataValidation sqref="I6 I7 I8 I9 I10 I11 I12 I13 I14 I15 I16 I17" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Capital Social,Lucros Acumulados"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -897,51 +987,51 @@
           <t>Cafeteria Grão de Ouro  |  Mês 1  |  valores em R$</t>
         </is>
       </c>
-      <c r="D1" s="9" t="inlineStr">
+      <c r="D1" s="11" t="inlineStr">
         <is>
           <t>Transações, por Número e Descrição</t>
         </is>
       </c>
     </row>
     <row r="2" ht="42" customHeight="1">
-      <c r="D2" s="10" t="inlineStr">
+      <c r="D2" s="12" t="inlineStr">
         <is>
           <t>Integralização de capital de R$ 80.000 em dinheiro</t>
         </is>
       </c>
-      <c r="E2" s="10" t="inlineStr">
+      <c r="E2" s="12" t="inlineStr">
         <is>
           <t>Compra à vista de máquina de espresso e mobiliário por R$ 30</t>
         </is>
       </c>
-      <c r="F2" s="10" t="inlineStr">
+      <c r="F2" s="12" t="inlineStr">
         <is>
           <t>Compra de café e insumos por R$ 24.000, metade à vista e met</t>
         </is>
       </c>
-      <c r="G2" s="10" t="inlineStr">
+      <c r="G2" s="12" t="inlineStr">
         <is>
           <t>Venda de metade do estoque por R$ 27.000 à vista (custo de R</t>
         </is>
       </c>
-      <c r="H2" s="10" t="inlineStr">
+      <c r="H2" s="12" t="inlineStr">
         <is>
           <t>Pagamento de salários e aluguel do mês, R$ 6.000 à vista</t>
         </is>
       </c>
-      <c r="I2" s="10" t="inlineStr">
+      <c r="I2" s="12" t="inlineStr">
         <is>
           <t>Pagamento de metade do que devia aos fornecedores</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="B3" s="11" t="inlineStr">
+      <c r="B3" s="13" t="inlineStr">
         <is>
           <t>Balanço Patrimonial</t>
         </is>
       </c>
-      <c r="C3" s="11" t="inlineStr">
+      <c r="C3" s="13" t="inlineStr">
         <is>
           <t>Balanço Inicial</t>
         </is>
@@ -964,21 +1054,21 @@
       <c r="I3" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="J3" s="11" t="inlineStr">
+      <c r="J3" s="13" t="inlineStr">
         <is>
           <t>Balanço Final</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="B4" s="12" t="inlineStr">
+      <c r="B4" s="14" t="inlineStr">
         <is>
           <t>ATIVO</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="B5" s="13" t="inlineStr">
+      <c r="B5" s="15" t="inlineStr">
         <is>
           <t>Ativo Circulante</t>
         </is>
@@ -990,18 +1080,18 @@
           <t>Caixa</t>
         </is>
       </c>
-      <c r="C6" s="14" t="n"/>
-      <c r="D6" s="6" t="n"/>
-      <c r="E6" s="6" t="n"/>
-      <c r="F6" s="6" t="n"/>
-      <c r="G6" s="6" t="n"/>
-      <c r="H6" s="6" t="n"/>
-      <c r="I6" s="6" t="n"/>
-      <c r="J6" s="15">
+      <c r="C6" s="16" t="n"/>
+      <c r="D6" s="9" t="n"/>
+      <c r="E6" s="9" t="n"/>
+      <c r="F6" s="9" t="n"/>
+      <c r="G6" s="9" t="n"/>
+      <c r="H6" s="9" t="n"/>
+      <c r="I6" s="9" t="n"/>
+      <c r="J6" s="17">
         <f>C6+SUM(D6:I6)</f>
         <v/>
       </c>
-      <c r="L6" s="16">
+      <c r="L6" s="18">
         <f>IF(COUNT(D6:I6)=0,"",IF(ABS(J6-Gabarito!J6)&lt;0.5,"✔","✗"))</f>
         <v/>
       </c>
@@ -1012,24 +1102,24 @@
           <t>Estoque</t>
         </is>
       </c>
-      <c r="C7" s="14" t="n"/>
-      <c r="D7" s="6" t="n"/>
-      <c r="E7" s="6" t="n"/>
-      <c r="F7" s="6" t="n"/>
-      <c r="G7" s="6" t="n"/>
-      <c r="H7" s="6" t="n"/>
-      <c r="I7" s="6" t="n"/>
-      <c r="J7" s="15">
+      <c r="C7" s="16" t="n"/>
+      <c r="D7" s="9" t="n"/>
+      <c r="E7" s="9" t="n"/>
+      <c r="F7" s="9" t="n"/>
+      <c r="G7" s="9" t="n"/>
+      <c r="H7" s="9" t="n"/>
+      <c r="I7" s="9" t="n"/>
+      <c r="J7" s="17">
         <f>C7+SUM(D7:I7)</f>
         <v/>
       </c>
-      <c r="L7" s="16">
+      <c r="L7" s="18">
         <f>IF(COUNT(D7:I7)=0,"",IF(ABS(J7-Gabarito!J7)&lt;0.5,"✔","✗"))</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="B8" s="13" t="inlineStr">
+      <c r="B8" s="15" t="inlineStr">
         <is>
           <t>Ativo Não Circulante</t>
         </is>
@@ -1041,70 +1131,70 @@
           <t>Imobilizado</t>
         </is>
       </c>
-      <c r="C9" s="14" t="n"/>
-      <c r="D9" s="6" t="n"/>
-      <c r="E9" s="6" t="n"/>
-      <c r="F9" s="6" t="n"/>
-      <c r="G9" s="6" t="n"/>
-      <c r="H9" s="6" t="n"/>
-      <c r="I9" s="6" t="n"/>
-      <c r="J9" s="15">
+      <c r="C9" s="16" t="n"/>
+      <c r="D9" s="9" t="n"/>
+      <c r="E9" s="9" t="n"/>
+      <c r="F9" s="9" t="n"/>
+      <c r="G9" s="9" t="n"/>
+      <c r="H9" s="9" t="n"/>
+      <c r="I9" s="9" t="n"/>
+      <c r="J9" s="17">
         <f>C9+SUM(D9:I9)</f>
         <v/>
       </c>
-      <c r="L9" s="16">
+      <c r="L9" s="18">
         <f>IF(COUNT(D9:I9)=0,"",IF(ABS(J9-Gabarito!J9)&lt;0.5,"✔","✗"))</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="B10" s="17" t="inlineStr">
+      <c r="B10" s="19" t="inlineStr">
         <is>
           <t xml:space="preserve">  Total do Ativo</t>
         </is>
       </c>
-      <c r="C10" s="18">
+      <c r="C10" s="20">
         <f>SUM(C6:C9)</f>
         <v/>
       </c>
-      <c r="D10" s="18">
+      <c r="D10" s="20">
         <f>SUM(D6:D9)</f>
         <v/>
       </c>
-      <c r="E10" s="18">
+      <c r="E10" s="20">
         <f>SUM(E6:E9)</f>
         <v/>
       </c>
-      <c r="F10" s="18">
+      <c r="F10" s="20">
         <f>SUM(F6:F9)</f>
         <v/>
       </c>
-      <c r="G10" s="18">
+      <c r="G10" s="20">
         <f>SUM(G6:G9)</f>
         <v/>
       </c>
-      <c r="H10" s="18">
+      <c r="H10" s="20">
         <f>SUM(H6:H9)</f>
         <v/>
       </c>
-      <c r="I10" s="18">
+      <c r="I10" s="20">
         <f>SUM(I6:I9)</f>
         <v/>
       </c>
-      <c r="J10" s="18">
+      <c r="J10" s="20">
         <f>SUM(J6:J9)</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="B11" s="12" t="inlineStr">
+      <c r="B11" s="14" t="inlineStr">
         <is>
           <t>PASSIVO E PATRIM. LÍQUIDO</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="B12" s="13" t="inlineStr">
+      <c r="B12" s="15" t="inlineStr">
         <is>
           <t>Passivo Circulante:</t>
         </is>
@@ -1116,24 +1206,24 @@
           <t>Contas a Pagar</t>
         </is>
       </c>
-      <c r="C13" s="14" t="n"/>
-      <c r="D13" s="6" t="n"/>
-      <c r="E13" s="6" t="n"/>
-      <c r="F13" s="6" t="n"/>
-      <c r="G13" s="6" t="n"/>
-      <c r="H13" s="6" t="n"/>
-      <c r="I13" s="6" t="n"/>
-      <c r="J13" s="15">
+      <c r="C13" s="16" t="n"/>
+      <c r="D13" s="9" t="n"/>
+      <c r="E13" s="9" t="n"/>
+      <c r="F13" s="9" t="n"/>
+      <c r="G13" s="9" t="n"/>
+      <c r="H13" s="9" t="n"/>
+      <c r="I13" s="9" t="n"/>
+      <c r="J13" s="17">
         <f>C13+SUM(D13:I13)</f>
         <v/>
       </c>
-      <c r="L13" s="16">
+      <c r="L13" s="18">
         <f>IF(COUNT(D13:I13)=0,"",IF(ABS(J13-Gabarito!J13)&lt;0.5,"✔","✗"))</f>
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="B14" s="13" t="inlineStr">
+      <c r="B14" s="15" t="inlineStr">
         <is>
           <t>Patrimônio Líquido:</t>
         </is>
@@ -1145,18 +1235,18 @@
           <t>Capital Social</t>
         </is>
       </c>
-      <c r="C15" s="14" t="n"/>
-      <c r="D15" s="6" t="n"/>
-      <c r="E15" s="6" t="n"/>
-      <c r="F15" s="6" t="n"/>
-      <c r="G15" s="6" t="n"/>
-      <c r="H15" s="6" t="n"/>
-      <c r="I15" s="6" t="n"/>
-      <c r="J15" s="15">
+      <c r="C15" s="16" t="n"/>
+      <c r="D15" s="9" t="n"/>
+      <c r="E15" s="9" t="n"/>
+      <c r="F15" s="9" t="n"/>
+      <c r="G15" s="9" t="n"/>
+      <c r="H15" s="9" t="n"/>
+      <c r="I15" s="9" t="n"/>
+      <c r="J15" s="17">
         <f>C15+SUM(D15:I15)</f>
         <v/>
       </c>
-      <c r="L15" s="16">
+      <c r="L15" s="18">
         <f>IF(COUNT(D15:I15)=0,"",IF(ABS(J15-Gabarito!J15)&lt;0.5,"✔","✗"))</f>
         <v/>
       </c>
@@ -1167,106 +1257,106 @@
           <t>Lucros Acumulados</t>
         </is>
       </c>
-      <c r="C16" s="14" t="n"/>
-      <c r="D16" s="6" t="n"/>
-      <c r="E16" s="6" t="n"/>
-      <c r="F16" s="6" t="n"/>
-      <c r="G16" s="6" t="n"/>
-      <c r="H16" s="6" t="n"/>
-      <c r="I16" s="6" t="n"/>
-      <c r="J16" s="15">
+      <c r="C16" s="16" t="n"/>
+      <c r="D16" s="9" t="n"/>
+      <c r="E16" s="9" t="n"/>
+      <c r="F16" s="9" t="n"/>
+      <c r="G16" s="9" t="n"/>
+      <c r="H16" s="9" t="n"/>
+      <c r="I16" s="9" t="n"/>
+      <c r="J16" s="17">
         <f>C16+SUM(D16:I16)</f>
         <v/>
       </c>
-      <c r="L16" s="16">
+      <c r="L16" s="18">
         <f>IF(COUNT(D16:I16)=0,"",IF(ABS(J16-Gabarito!J16)&lt;0.5,"✔","✗"))</f>
         <v/>
       </c>
     </row>
     <row r="17">
-      <c r="B17" s="17" t="inlineStr">
+      <c r="B17" s="19" t="inlineStr">
         <is>
           <t>Total Passivo e Patrim. Líquido</t>
         </is>
       </c>
-      <c r="C17" s="18">
+      <c r="C17" s="20">
         <f>SUM(C12:C16)</f>
         <v/>
       </c>
-      <c r="D17" s="18">
+      <c r="D17" s="20">
         <f>SUM(D12:D16)</f>
         <v/>
       </c>
-      <c r="E17" s="18">
+      <c r="E17" s="20">
         <f>SUM(E12:E16)</f>
         <v/>
       </c>
-      <c r="F17" s="18">
+      <c r="F17" s="20">
         <f>SUM(F12:F16)</f>
         <v/>
       </c>
-      <c r="G17" s="18">
+      <c r="G17" s="20">
         <f>SUM(G12:G16)</f>
         <v/>
       </c>
-      <c r="H17" s="18">
+      <c r="H17" s="20">
         <f>SUM(H12:H16)</f>
         <v/>
       </c>
-      <c r="I17" s="18">
+      <c r="I17" s="20">
         <f>SUM(I12:I16)</f>
         <v/>
       </c>
-      <c r="J17" s="18">
+      <c r="J17" s="20">
         <f>SUM(J12:J16)</f>
         <v/>
       </c>
     </row>
     <row r="19">
-      <c r="B19" s="19" t="inlineStr">
+      <c r="B19" s="21" t="inlineStr">
         <is>
           <t>Diferença, se houver (tem que dar zero)</t>
         </is>
       </c>
-      <c r="C19" s="15">
+      <c r="C19" s="17">
         <f>C10-C17</f>
         <v/>
       </c>
-      <c r="D19" s="15">
+      <c r="D19" s="17">
         <f>D10-D17</f>
         <v/>
       </c>
-      <c r="E19" s="15">
+      <c r="E19" s="17">
         <f>E10-E17</f>
         <v/>
       </c>
-      <c r="F19" s="15">
+      <c r="F19" s="17">
         <f>F10-F17</f>
         <v/>
       </c>
-      <c r="G19" s="15">
+      <c r="G19" s="17">
         <f>G10-G17</f>
         <v/>
       </c>
-      <c r="H19" s="15">
+      <c r="H19" s="17">
         <f>H10-H17</f>
         <v/>
       </c>
-      <c r="I19" s="15">
+      <c r="I19" s="17">
         <f>I10-I17</f>
         <v/>
       </c>
-      <c r="J19" s="15">
+      <c r="J19" s="17">
         <f>J10-J17</f>
         <v/>
       </c>
-      <c r="L19" s="17">
+      <c r="L19" s="19">
         <f>IF(J19=0,"✔ fecha","✗ não fecha")</f>
         <v/>
       </c>
     </row>
     <row r="21">
-      <c r="B21" s="11" t="inlineStr">
+      <c r="B21" s="13" t="inlineStr">
         <is>
           <t>Demonstração do Resultado</t>
         </is>
@@ -1289,12 +1379,12 @@
       <c r="I21" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="J21" s="11" t="inlineStr">
+      <c r="J21" s="13" t="inlineStr">
         <is>
           <t>Mês 1</t>
         </is>
       </c>
-      <c r="L21" s="20" t="inlineStr">
+      <c r="L21" s="22" t="inlineStr">
         <is>
           <t>Check</t>
         </is>
@@ -1306,17 +1396,17 @@
           <t>Receita de Vendas</t>
         </is>
       </c>
-      <c r="D22" s="6" t="n"/>
-      <c r="E22" s="6" t="n"/>
-      <c r="F22" s="6" t="n"/>
-      <c r="G22" s="6" t="n"/>
-      <c r="H22" s="6" t="n"/>
-      <c r="I22" s="6" t="n"/>
-      <c r="J22" s="15">
+      <c r="D22" s="9" t="n"/>
+      <c r="E22" s="9" t="n"/>
+      <c r="F22" s="9" t="n"/>
+      <c r="G22" s="9" t="n"/>
+      <c r="H22" s="9" t="n"/>
+      <c r="I22" s="9" t="n"/>
+      <c r="J22" s="17">
         <f>SUM(D22:I22)</f>
         <v/>
       </c>
-      <c r="L22" s="16">
+      <c r="L22" s="18">
         <f>IF(COUNT(D22:I22)=0,"",IF(ABS(J22-Gabarito!J22)&lt;0.5,"✔","✗"))</f>
         <v/>
       </c>
@@ -1327,52 +1417,52 @@
           <t>(-) Custo das Mercadorias Vendidas</t>
         </is>
       </c>
-      <c r="D23" s="6" t="n"/>
-      <c r="E23" s="6" t="n"/>
-      <c r="F23" s="6" t="n"/>
-      <c r="G23" s="6" t="n"/>
-      <c r="H23" s="6" t="n"/>
-      <c r="I23" s="6" t="n"/>
-      <c r="J23" s="15">
+      <c r="D23" s="9" t="n"/>
+      <c r="E23" s="9" t="n"/>
+      <c r="F23" s="9" t="n"/>
+      <c r="G23" s="9" t="n"/>
+      <c r="H23" s="9" t="n"/>
+      <c r="I23" s="9" t="n"/>
+      <c r="J23" s="17">
         <f>SUM(D23:I23)</f>
         <v/>
       </c>
-      <c r="L23" s="16">
+      <c r="L23" s="18">
         <f>IF(COUNT(D23:I23)=0,"",IF(ABS(J23-Gabarito!J23)&lt;0.5,"✔","✗"))</f>
         <v/>
       </c>
     </row>
     <row r="24">
-      <c r="B24" s="17" t="inlineStr">
+      <c r="B24" s="19" t="inlineStr">
         <is>
           <t xml:space="preserve">     (=) Lucro Bruto</t>
         </is>
       </c>
-      <c r="D24" s="18">
+      <c r="D24" s="20">
         <f>SUM(D22:D23)</f>
         <v/>
       </c>
-      <c r="E24" s="18">
+      <c r="E24" s="20">
         <f>SUM(E22:E23)</f>
         <v/>
       </c>
-      <c r="F24" s="18">
+      <c r="F24" s="20">
         <f>SUM(F22:F23)</f>
         <v/>
       </c>
-      <c r="G24" s="18">
+      <c r="G24" s="20">
         <f>SUM(G22:G23)</f>
         <v/>
       </c>
-      <c r="H24" s="18">
+      <c r="H24" s="20">
         <f>SUM(H22:H23)</f>
         <v/>
       </c>
-      <c r="I24" s="18">
+      <c r="I24" s="20">
         <f>SUM(I22:I23)</f>
         <v/>
       </c>
-      <c r="J24" s="18">
+      <c r="J24" s="20">
         <f>SUM(J22:J23)</f>
         <v/>
       </c>
@@ -1383,58 +1473,58 @@
           <t>(-) Despesas Operacionais</t>
         </is>
       </c>
-      <c r="D25" s="6" t="n"/>
-      <c r="E25" s="6" t="n"/>
-      <c r="F25" s="6" t="n"/>
-      <c r="G25" s="6" t="n"/>
-      <c r="H25" s="6" t="n"/>
-      <c r="I25" s="6" t="n"/>
-      <c r="J25" s="15">
+      <c r="D25" s="9" t="n"/>
+      <c r="E25" s="9" t="n"/>
+      <c r="F25" s="9" t="n"/>
+      <c r="G25" s="9" t="n"/>
+      <c r="H25" s="9" t="n"/>
+      <c r="I25" s="9" t="n"/>
+      <c r="J25" s="17">
         <f>SUM(D25:I25)</f>
         <v/>
       </c>
-      <c r="L25" s="16">
+      <c r="L25" s="18">
         <f>IF(COUNT(D25:I25)=0,"",IF(ABS(J25-Gabarito!J25)&lt;0.5,"✔","✗"))</f>
         <v/>
       </c>
     </row>
     <row r="26">
-      <c r="B26" s="17" t="inlineStr">
+      <c r="B26" s="19" t="inlineStr">
         <is>
           <t xml:space="preserve">     (=) EBIT e Lucro Líquido</t>
         </is>
       </c>
-      <c r="D26" s="18">
+      <c r="D26" s="20">
         <f>SUM(D24:D25)</f>
         <v/>
       </c>
-      <c r="E26" s="18">
+      <c r="E26" s="20">
         <f>SUM(E24:E25)</f>
         <v/>
       </c>
-      <c r="F26" s="18">
+      <c r="F26" s="20">
         <f>SUM(F24:F25)</f>
         <v/>
       </c>
-      <c r="G26" s="18">
+      <c r="G26" s="20">
         <f>SUM(G24:G25)</f>
         <v/>
       </c>
-      <c r="H26" s="18">
+      <c r="H26" s="20">
         <f>SUM(H24:H25)</f>
         <v/>
       </c>
-      <c r="I26" s="18">
+      <c r="I26" s="20">
         <f>SUM(I24:I25)</f>
         <v/>
       </c>
-      <c r="J26" s="18">
+      <c r="J26" s="20">
         <f>SUM(J24:J25)</f>
         <v/>
       </c>
     </row>
     <row r="28">
-      <c r="B28" s="11" t="inlineStr">
+      <c r="B28" s="13" t="inlineStr">
         <is>
           <t>Demonstração dos Fluxos de Caixa</t>
         </is>
@@ -1457,43 +1547,43 @@
       <c r="I28" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="J28" s="11" t="inlineStr">
+      <c r="J28" s="13" t="inlineStr">
         <is>
           <t>Mês 1</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="B29" s="17" t="inlineStr">
+      <c r="B29" s="19" t="inlineStr">
         <is>
           <t>OPERAÇÕES</t>
         </is>
       </c>
-      <c r="D29" s="18">
+      <c r="D29" s="20">
         <f>SUM(D30:D32)</f>
         <v/>
       </c>
-      <c r="E29" s="18">
+      <c r="E29" s="20">
         <f>SUM(E30:E32)</f>
         <v/>
       </c>
-      <c r="F29" s="18">
+      <c r="F29" s="20">
         <f>SUM(F30:F32)</f>
         <v/>
       </c>
-      <c r="G29" s="18">
+      <c r="G29" s="20">
         <f>SUM(G30:G32)</f>
         <v/>
       </c>
-      <c r="H29" s="18">
+      <c r="H29" s="20">
         <f>SUM(H30:H32)</f>
         <v/>
       </c>
-      <c r="I29" s="18">
+      <c r="I29" s="20">
         <f>SUM(I30:I32)</f>
         <v/>
       </c>
-      <c r="J29" s="18">
+      <c r="J29" s="20">
         <f>SUM(J30:J32)</f>
         <v/>
       </c>
@@ -1504,17 +1594,17 @@
           <t>Recebimentos de Clientes</t>
         </is>
       </c>
-      <c r="D30" s="6" t="n"/>
-      <c r="E30" s="6" t="n"/>
-      <c r="F30" s="6" t="n"/>
-      <c r="G30" s="6" t="n"/>
-      <c r="H30" s="6" t="n"/>
-      <c r="I30" s="6" t="n"/>
-      <c r="J30" s="15">
+      <c r="D30" s="9" t="n"/>
+      <c r="E30" s="9" t="n"/>
+      <c r="F30" s="9" t="n"/>
+      <c r="G30" s="9" t="n"/>
+      <c r="H30" s="9" t="n"/>
+      <c r="I30" s="9" t="n"/>
+      <c r="J30" s="17">
         <f>SUM(D30:I30)</f>
         <v/>
       </c>
-      <c r="L30" s="16">
+      <c r="L30" s="18">
         <f>IF(COUNT(D30:I30)=0,"",IF(ABS(J30-Gabarito!J30)&lt;0.5,"✔","✗"))</f>
         <v/>
       </c>
@@ -1525,17 +1615,17 @@
           <t>Pagamentos a Fornecedores</t>
         </is>
       </c>
-      <c r="D31" s="6" t="n"/>
-      <c r="E31" s="6" t="n"/>
-      <c r="F31" s="6" t="n"/>
-      <c r="G31" s="6" t="n"/>
-      <c r="H31" s="6" t="n"/>
-      <c r="I31" s="6" t="n"/>
-      <c r="J31" s="15">
+      <c r="D31" s="9" t="n"/>
+      <c r="E31" s="9" t="n"/>
+      <c r="F31" s="9" t="n"/>
+      <c r="G31" s="9" t="n"/>
+      <c r="H31" s="9" t="n"/>
+      <c r="I31" s="9" t="n"/>
+      <c r="J31" s="17">
         <f>SUM(D31:I31)</f>
         <v/>
       </c>
-      <c r="L31" s="16">
+      <c r="L31" s="18">
         <f>IF(COUNT(D31:I31)=0,"",IF(ABS(J31-Gabarito!J31)&lt;0.5,"✔","✗"))</f>
         <v/>
       </c>
@@ -1546,52 +1636,52 @@
           <t>Pagamentos de Despesas</t>
         </is>
       </c>
-      <c r="D32" s="6" t="n"/>
-      <c r="E32" s="6" t="n"/>
-      <c r="F32" s="6" t="n"/>
-      <c r="G32" s="6" t="n"/>
-      <c r="H32" s="6" t="n"/>
-      <c r="I32" s="6" t="n"/>
-      <c r="J32" s="15">
+      <c r="D32" s="9" t="n"/>
+      <c r="E32" s="9" t="n"/>
+      <c r="F32" s="9" t="n"/>
+      <c r="G32" s="9" t="n"/>
+      <c r="H32" s="9" t="n"/>
+      <c r="I32" s="9" t="n"/>
+      <c r="J32" s="17">
         <f>SUM(D32:I32)</f>
         <v/>
       </c>
-      <c r="L32" s="16">
+      <c r="L32" s="18">
         <f>IF(COUNT(D32:I32)=0,"",IF(ABS(J32-Gabarito!J32)&lt;0.5,"✔","✗"))</f>
         <v/>
       </c>
     </row>
     <row r="33">
-      <c r="B33" s="17" t="inlineStr">
+      <c r="B33" s="19" t="inlineStr">
         <is>
           <t>INVESTIMENTOS</t>
         </is>
       </c>
-      <c r="D33" s="18">
+      <c r="D33" s="20">
         <f>SUM(D34:D34)</f>
         <v/>
       </c>
-      <c r="E33" s="18">
+      <c r="E33" s="20">
         <f>SUM(E34:E34)</f>
         <v/>
       </c>
-      <c r="F33" s="18">
+      <c r="F33" s="20">
         <f>SUM(F34:F34)</f>
         <v/>
       </c>
-      <c r="G33" s="18">
+      <c r="G33" s="20">
         <f>SUM(G34:G34)</f>
         <v/>
       </c>
-      <c r="H33" s="18">
+      <c r="H33" s="20">
         <f>SUM(H34:H34)</f>
         <v/>
       </c>
-      <c r="I33" s="18">
+      <c r="I33" s="20">
         <f>SUM(I34:I34)</f>
         <v/>
       </c>
-      <c r="J33" s="18">
+      <c r="J33" s="20">
         <f>SUM(J34:J34)</f>
         <v/>
       </c>
@@ -1602,52 +1692,52 @@
           <t>Aquisição de Imobilizado</t>
         </is>
       </c>
-      <c r="D34" s="6" t="n"/>
-      <c r="E34" s="6" t="n"/>
-      <c r="F34" s="6" t="n"/>
-      <c r="G34" s="6" t="n"/>
-      <c r="H34" s="6" t="n"/>
-      <c r="I34" s="6" t="n"/>
-      <c r="J34" s="15">
+      <c r="D34" s="9" t="n"/>
+      <c r="E34" s="9" t="n"/>
+      <c r="F34" s="9" t="n"/>
+      <c r="G34" s="9" t="n"/>
+      <c r="H34" s="9" t="n"/>
+      <c r="I34" s="9" t="n"/>
+      <c r="J34" s="17">
         <f>SUM(D34:I34)</f>
         <v/>
       </c>
-      <c r="L34" s="16">
+      <c r="L34" s="18">
         <f>IF(COUNT(D34:I34)=0,"",IF(ABS(J34-Gabarito!J34)&lt;0.5,"✔","✗"))</f>
         <v/>
       </c>
     </row>
     <row r="35">
-      <c r="B35" s="17" t="inlineStr">
+      <c r="B35" s="19" t="inlineStr">
         <is>
           <t>FINANCIAMENTOS</t>
         </is>
       </c>
-      <c r="D35" s="18">
+      <c r="D35" s="20">
         <f>SUM(D36:D36)</f>
         <v/>
       </c>
-      <c r="E35" s="18">
+      <c r="E35" s="20">
         <f>SUM(E36:E36)</f>
         <v/>
       </c>
-      <c r="F35" s="18">
+      <c r="F35" s="20">
         <f>SUM(F36:F36)</f>
         <v/>
       </c>
-      <c r="G35" s="18">
+      <c r="G35" s="20">
         <f>SUM(G36:G36)</f>
         <v/>
       </c>
-      <c r="H35" s="18">
+      <c r="H35" s="20">
         <f>SUM(H36:H36)</f>
         <v/>
       </c>
-      <c r="I35" s="18">
+      <c r="I35" s="20">
         <f>SUM(I36:I36)</f>
         <v/>
       </c>
-      <c r="J35" s="18">
+      <c r="J35" s="20">
         <f>SUM(J36:J36)</f>
         <v/>
       </c>
@@ -1658,52 +1748,52 @@
           <t>Ingresso de Capital</t>
         </is>
       </c>
-      <c r="D36" s="6" t="n"/>
-      <c r="E36" s="6" t="n"/>
-      <c r="F36" s="6" t="n"/>
-      <c r="G36" s="6" t="n"/>
-      <c r="H36" s="6" t="n"/>
-      <c r="I36" s="6" t="n"/>
-      <c r="J36" s="15">
+      <c r="D36" s="9" t="n"/>
+      <c r="E36" s="9" t="n"/>
+      <c r="F36" s="9" t="n"/>
+      <c r="G36" s="9" t="n"/>
+      <c r="H36" s="9" t="n"/>
+      <c r="I36" s="9" t="n"/>
+      <c r="J36" s="17">
         <f>SUM(D36:I36)</f>
         <v/>
       </c>
-      <c r="L36" s="16">
+      <c r="L36" s="18">
         <f>IF(COUNT(D36:I36)=0,"",IF(ABS(J36-Gabarito!J36)&lt;0.5,"✔","✗"))</f>
         <v/>
       </c>
     </row>
     <row r="37">
-      <c r="B37" s="17" t="inlineStr">
+      <c r="B37" s="19" t="inlineStr">
         <is>
           <t>VARIAÇÃO NO CAIXA</t>
         </is>
       </c>
-      <c r="D37" s="18">
+      <c r="D37" s="20">
         <f>D29+D33+D35</f>
         <v/>
       </c>
-      <c r="E37" s="18">
+      <c r="E37" s="20">
         <f>E29+E33+E35</f>
         <v/>
       </c>
-      <c r="F37" s="18">
+      <c r="F37" s="20">
         <f>F29+F33+F35</f>
         <v/>
       </c>
-      <c r="G37" s="18">
+      <c r="G37" s="20">
         <f>G29+G33+G35</f>
         <v/>
       </c>
-      <c r="H37" s="18">
+      <c r="H37" s="20">
         <f>H29+H33+H35</f>
         <v/>
       </c>
-      <c r="I37" s="18">
+      <c r="I37" s="20">
         <f>I29+I33+I35</f>
         <v/>
       </c>
-      <c r="J37" s="18">
+      <c r="J37" s="20">
         <f>J29+J33+J35</f>
         <v/>
       </c>
@@ -1714,38 +1804,38 @@
           <t xml:space="preserve">    Saldo inicial de caixa</t>
         </is>
       </c>
-      <c r="J38" s="14" t="n">
+      <c r="J38" s="16" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="39">
-      <c r="B39" s="17" t="inlineStr">
+      <c r="B39" s="19" t="inlineStr">
         <is>
           <t xml:space="preserve">    Saldo final de caixa</t>
         </is>
       </c>
-      <c r="J39" s="15">
+      <c r="J39" s="17">
         <f>J38+J37</f>
         <v/>
       </c>
     </row>
     <row r="41">
-      <c r="B41" s="19" t="inlineStr">
+      <c r="B41" s="21" t="inlineStr">
         <is>
           <t>Caixa final da DFC menos Caixa do BP (tem que dar zero)</t>
         </is>
       </c>
-      <c r="J41" s="15">
+      <c r="J41" s="17">
         <f>J39-J6</f>
         <v/>
       </c>
-      <c r="L41" s="17">
+      <c r="L41" s="19">
         <f>IF(J41=0,"✔ amarra","✗ não amarra")</f>
         <v/>
       </c>
     </row>
     <row r="43">
-      <c r="B43" s="11" t="inlineStr">
+      <c r="B43" s="13" t="inlineStr">
         <is>
           <t>Indicadores (automáticos)</t>
         </is>
@@ -1757,7 +1847,7 @@
           <t>Margem bruta</t>
         </is>
       </c>
-      <c r="J44" s="21">
+      <c r="J44" s="23">
         <f>IF(J22=0,"",J24/J22)</f>
         <v/>
       </c>
@@ -1768,7 +1858,7 @@
           <t>Margem líquida</t>
         </is>
       </c>
-      <c r="J45" s="21">
+      <c r="J45" s="23">
         <f>IF(J22=0,"",J26/J22)</f>
         <v/>
       </c>
@@ -1779,7 +1869,7 @@
           <t>% financiado por capital próprio (PL / Ativo)</t>
         </is>
       </c>
-      <c r="J46" s="21">
+      <c r="J46" s="23">
         <f>IF(J10=0,"",SUM(J15:J16)/J10)</f>
         <v/>
       </c>
@@ -1790,7 +1880,7 @@
           <t>ROE (LL / PL final)</t>
         </is>
       </c>
-      <c r="J47" s="21">
+      <c r="J47" s="23">
         <f>IF(SUM(J15:J16)=0,"",J26/SUM(J15:J16))</f>
         <v/>
       </c>
@@ -1829,51 +1919,51 @@
           <t>Cafeteria Grão de Ouro  |  Mês 1  |  valores em R$</t>
         </is>
       </c>
-      <c r="D1" s="9" t="inlineStr">
+      <c r="D1" s="11" t="inlineStr">
         <is>
           <t>Transações, por Número e Descrição</t>
         </is>
       </c>
     </row>
     <row r="2" ht="42" customHeight="1">
-      <c r="D2" s="10" t="inlineStr">
+      <c r="D2" s="12" t="inlineStr">
         <is>
           <t>Integralização de capital de R$ 80.000 em dinheiro</t>
         </is>
       </c>
-      <c r="E2" s="10" t="inlineStr">
+      <c r="E2" s="12" t="inlineStr">
         <is>
           <t>Compra à vista de máquina de espresso e mobiliário por R$ 30</t>
         </is>
       </c>
-      <c r="F2" s="10" t="inlineStr">
+      <c r="F2" s="12" t="inlineStr">
         <is>
           <t>Compra de café e insumos por R$ 24.000, metade à vista e met</t>
         </is>
       </c>
-      <c r="G2" s="10" t="inlineStr">
+      <c r="G2" s="12" t="inlineStr">
         <is>
           <t>Venda de metade do estoque por R$ 27.000 à vista (custo de R</t>
         </is>
       </c>
-      <c r="H2" s="10" t="inlineStr">
+      <c r="H2" s="12" t="inlineStr">
         <is>
           <t>Pagamento de salários e aluguel do mês, R$ 6.000 à vista</t>
         </is>
       </c>
-      <c r="I2" s="10" t="inlineStr">
+      <c r="I2" s="12" t="inlineStr">
         <is>
           <t>Pagamento de metade do que devia aos fornecedores</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="B3" s="11" t="inlineStr">
+      <c r="B3" s="13" t="inlineStr">
         <is>
           <t>Balanço Patrimonial</t>
         </is>
       </c>
-      <c r="C3" s="11" t="inlineStr">
+      <c r="C3" s="13" t="inlineStr">
         <is>
           <t>Balanço Inicial</t>
         </is>
@@ -1896,21 +1986,21 @@
       <c r="I3" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="J3" s="11" t="inlineStr">
+      <c r="J3" s="13" t="inlineStr">
         <is>
           <t>Balanço Final</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="B4" s="12" t="inlineStr">
+      <c r="B4" s="14" t="inlineStr">
         <is>
           <t>ATIVO</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="B5" s="13" t="inlineStr">
+      <c r="B5" s="15" t="inlineStr">
         <is>
           <t>Ativo Circulante</t>
         </is>
@@ -1922,26 +2012,26 @@
           <t>Caixa</t>
         </is>
       </c>
-      <c r="C6" s="14" t="n"/>
-      <c r="D6" s="6" t="n">
+      <c r="C6" s="16" t="n"/>
+      <c r="D6" s="9" t="n">
         <v>80000</v>
       </c>
-      <c r="E6" s="6" t="n">
+      <c r="E6" s="9" t="n">
         <v>-30000</v>
       </c>
-      <c r="F6" s="6" t="n">
+      <c r="F6" s="9" t="n">
         <v>-12000</v>
       </c>
-      <c r="G6" s="6" t="n">
+      <c r="G6" s="9" t="n">
         <v>27000</v>
       </c>
-      <c r="H6" s="6" t="n">
+      <c r="H6" s="9" t="n">
         <v>-6000</v>
       </c>
-      <c r="I6" s="6" t="n">
+      <c r="I6" s="9" t="n">
         <v>-6000</v>
       </c>
-      <c r="J6" s="15">
+      <c r="J6" s="17">
         <f>C6+SUM(D6:I6)</f>
         <v/>
       </c>
@@ -1952,24 +2042,24 @@
           <t>Estoque</t>
         </is>
       </c>
-      <c r="C7" s="14" t="n"/>
-      <c r="D7" s="6" t="n"/>
-      <c r="E7" s="6" t="n"/>
-      <c r="F7" s="6" t="n">
+      <c r="C7" s="16" t="n"/>
+      <c r="D7" s="9" t="n"/>
+      <c r="E7" s="9" t="n"/>
+      <c r="F7" s="9" t="n">
         <v>24000</v>
       </c>
-      <c r="G7" s="6" t="n">
+      <c r="G7" s="9" t="n">
         <v>-12000</v>
       </c>
-      <c r="H7" s="6" t="n"/>
-      <c r="I7" s="6" t="n"/>
-      <c r="J7" s="15">
+      <c r="H7" s="9" t="n"/>
+      <c r="I7" s="9" t="n"/>
+      <c r="J7" s="17">
         <f>C7+SUM(D7:I7)</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="B8" s="13" t="inlineStr">
+      <c r="B8" s="15" t="inlineStr">
         <is>
           <t>Ativo Não Circulante</t>
         </is>
@@ -1981,68 +2071,68 @@
           <t>Imobilizado</t>
         </is>
       </c>
-      <c r="C9" s="14" t="n"/>
-      <c r="D9" s="6" t="n"/>
-      <c r="E9" s="6" t="n">
+      <c r="C9" s="16" t="n"/>
+      <c r="D9" s="9" t="n"/>
+      <c r="E9" s="9" t="n">
         <v>30000</v>
       </c>
-      <c r="F9" s="6" t="n"/>
-      <c r="G9" s="6" t="n"/>
-      <c r="H9" s="6" t="n"/>
-      <c r="I9" s="6" t="n"/>
-      <c r="J9" s="15">
+      <c r="F9" s="9" t="n"/>
+      <c r="G9" s="9" t="n"/>
+      <c r="H9" s="9" t="n"/>
+      <c r="I9" s="9" t="n"/>
+      <c r="J9" s="17">
         <f>C9+SUM(D9:I9)</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="B10" s="17" t="inlineStr">
+      <c r="B10" s="19" t="inlineStr">
         <is>
           <t xml:space="preserve">  Total do Ativo</t>
         </is>
       </c>
-      <c r="C10" s="18">
+      <c r="C10" s="20">
         <f>SUM(C6:C9)</f>
         <v/>
       </c>
-      <c r="D10" s="18">
+      <c r="D10" s="20">
         <f>SUM(D6:D9)</f>
         <v/>
       </c>
-      <c r="E10" s="18">
+      <c r="E10" s="20">
         <f>SUM(E6:E9)</f>
         <v/>
       </c>
-      <c r="F10" s="18">
+      <c r="F10" s="20">
         <f>SUM(F6:F9)</f>
         <v/>
       </c>
-      <c r="G10" s="18">
+      <c r="G10" s="20">
         <f>SUM(G6:G9)</f>
         <v/>
       </c>
-      <c r="H10" s="18">
+      <c r="H10" s="20">
         <f>SUM(H6:H9)</f>
         <v/>
       </c>
-      <c r="I10" s="18">
+      <c r="I10" s="20">
         <f>SUM(I6:I9)</f>
         <v/>
       </c>
-      <c r="J10" s="18">
+      <c r="J10" s="20">
         <f>SUM(J6:J9)</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="B11" s="12" t="inlineStr">
+      <c r="B11" s="14" t="inlineStr">
         <is>
           <t>PASSIVO E PATRIM. LÍQUIDO</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="B12" s="13" t="inlineStr">
+      <c r="B12" s="15" t="inlineStr">
         <is>
           <t>Passivo Circulante:</t>
         </is>
@@ -2054,24 +2144,24 @@
           <t>Contas a Pagar</t>
         </is>
       </c>
-      <c r="C13" s="14" t="n"/>
-      <c r="D13" s="6" t="n"/>
-      <c r="E13" s="6" t="n"/>
-      <c r="F13" s="6" t="n">
+      <c r="C13" s="16" t="n"/>
+      <c r="D13" s="9" t="n"/>
+      <c r="E13" s="9" t="n"/>
+      <c r="F13" s="9" t="n">
         <v>12000</v>
       </c>
-      <c r="G13" s="6" t="n"/>
-      <c r="H13" s="6" t="n"/>
-      <c r="I13" s="6" t="n">
+      <c r="G13" s="9" t="n"/>
+      <c r="H13" s="9" t="n"/>
+      <c r="I13" s="9" t="n">
         <v>-6000</v>
       </c>
-      <c r="J13" s="15">
+      <c r="J13" s="17">
         <f>C13+SUM(D13:I13)</f>
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="B14" s="13" t="inlineStr">
+      <c r="B14" s="15" t="inlineStr">
         <is>
           <t>Patrimônio Líquido:</t>
         </is>
@@ -2083,16 +2173,16 @@
           <t>Capital Social</t>
         </is>
       </c>
-      <c r="C15" s="14" t="n"/>
-      <c r="D15" s="6" t="n">
+      <c r="C15" s="16" t="n"/>
+      <c r="D15" s="9" t="n">
         <v>80000</v>
       </c>
-      <c r="E15" s="6" t="n"/>
-      <c r="F15" s="6" t="n"/>
-      <c r="G15" s="6" t="n"/>
-      <c r="H15" s="6" t="n"/>
-      <c r="I15" s="6" t="n"/>
-      <c r="J15" s="15">
+      <c r="E15" s="9" t="n"/>
+      <c r="F15" s="9" t="n"/>
+      <c r="G15" s="9" t="n"/>
+      <c r="H15" s="9" t="n"/>
+      <c r="I15" s="9" t="n"/>
+      <c r="J15" s="17">
         <f>C15+SUM(D15:I15)</f>
         <v/>
       </c>
@@ -2103,102 +2193,102 @@
           <t>Lucros Acumulados</t>
         </is>
       </c>
-      <c r="C16" s="14" t="n"/>
-      <c r="D16" s="6" t="n"/>
-      <c r="E16" s="6" t="n"/>
-      <c r="F16" s="6" t="n"/>
-      <c r="G16" s="6" t="n">
+      <c r="C16" s="16" t="n"/>
+      <c r="D16" s="9" t="n"/>
+      <c r="E16" s="9" t="n"/>
+      <c r="F16" s="9" t="n"/>
+      <c r="G16" s="9" t="n">
         <v>15000</v>
       </c>
-      <c r="H16" s="6" t="n">
+      <c r="H16" s="9" t="n">
         <v>-6000</v>
       </c>
-      <c r="I16" s="6" t="n"/>
-      <c r="J16" s="15">
+      <c r="I16" s="9" t="n"/>
+      <c r="J16" s="17">
         <f>C16+SUM(D16:I16)</f>
         <v/>
       </c>
     </row>
     <row r="17">
-      <c r="B17" s="17" t="inlineStr">
+      <c r="B17" s="19" t="inlineStr">
         <is>
           <t>Total Passivo e Patrim. Líquido</t>
         </is>
       </c>
-      <c r="C17" s="18">
+      <c r="C17" s="20">
         <f>SUM(C12:C16)</f>
         <v/>
       </c>
-      <c r="D17" s="18">
+      <c r="D17" s="20">
         <f>SUM(D12:D16)</f>
         <v/>
       </c>
-      <c r="E17" s="18">
+      <c r="E17" s="20">
         <f>SUM(E12:E16)</f>
         <v/>
       </c>
-      <c r="F17" s="18">
+      <c r="F17" s="20">
         <f>SUM(F12:F16)</f>
         <v/>
       </c>
-      <c r="G17" s="18">
+      <c r="G17" s="20">
         <f>SUM(G12:G16)</f>
         <v/>
       </c>
-      <c r="H17" s="18">
+      <c r="H17" s="20">
         <f>SUM(H12:H16)</f>
         <v/>
       </c>
-      <c r="I17" s="18">
+      <c r="I17" s="20">
         <f>SUM(I12:I16)</f>
         <v/>
       </c>
-      <c r="J17" s="18">
+      <c r="J17" s="20">
         <f>SUM(J12:J16)</f>
         <v/>
       </c>
     </row>
     <row r="19">
-      <c r="B19" s="19" t="inlineStr">
+      <c r="B19" s="21" t="inlineStr">
         <is>
           <t>Diferença, se houver (tem que dar zero)</t>
         </is>
       </c>
-      <c r="C19" s="15">
+      <c r="C19" s="17">
         <f>C10-C17</f>
         <v/>
       </c>
-      <c r="D19" s="15">
+      <c r="D19" s="17">
         <f>D10-D17</f>
         <v/>
       </c>
-      <c r="E19" s="15">
+      <c r="E19" s="17">
         <f>E10-E17</f>
         <v/>
       </c>
-      <c r="F19" s="15">
+      <c r="F19" s="17">
         <f>F10-F17</f>
         <v/>
       </c>
-      <c r="G19" s="15">
+      <c r="G19" s="17">
         <f>G10-G17</f>
         <v/>
       </c>
-      <c r="H19" s="15">
+      <c r="H19" s="17">
         <f>H10-H17</f>
         <v/>
       </c>
-      <c r="I19" s="15">
+      <c r="I19" s="17">
         <f>I10-I17</f>
         <v/>
       </c>
-      <c r="J19" s="15">
+      <c r="J19" s="17">
         <f>J10-J17</f>
         <v/>
       </c>
     </row>
     <row r="21">
-      <c r="B21" s="11" t="inlineStr">
+      <c r="B21" s="13" t="inlineStr">
         <is>
           <t>Demonstração do Resultado</t>
         </is>
@@ -2221,12 +2311,12 @@
       <c r="I21" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="J21" s="11" t="inlineStr">
+      <c r="J21" s="13" t="inlineStr">
         <is>
           <t>Mês 1</t>
         </is>
       </c>
-      <c r="L21" s="20" t="inlineStr">
+      <c r="L21" s="22" t="inlineStr">
         <is>
           <t>Check</t>
         </is>
@@ -2238,15 +2328,15 @@
           <t>Receita de Vendas</t>
         </is>
       </c>
-      <c r="D22" s="6" t="n"/>
-      <c r="E22" s="6" t="n"/>
-      <c r="F22" s="6" t="n"/>
-      <c r="G22" s="6" t="n">
+      <c r="D22" s="9" t="n"/>
+      <c r="E22" s="9" t="n"/>
+      <c r="F22" s="9" t="n"/>
+      <c r="G22" s="9" t="n">
         <v>27000</v>
       </c>
-      <c r="H22" s="6" t="n"/>
-      <c r="I22" s="6" t="n"/>
-      <c r="J22" s="15">
+      <c r="H22" s="9" t="n"/>
+      <c r="I22" s="9" t="n"/>
+      <c r="J22" s="17">
         <f>SUM(D22:I22)</f>
         <v/>
       </c>
@@ -2257,50 +2347,50 @@
           <t>(-) Custo das Mercadorias Vendidas</t>
         </is>
       </c>
-      <c r="D23" s="6" t="n"/>
-      <c r="E23" s="6" t="n"/>
-      <c r="F23" s="6" t="n"/>
-      <c r="G23" s="6" t="n">
+      <c r="D23" s="9" t="n"/>
+      <c r="E23" s="9" t="n"/>
+      <c r="F23" s="9" t="n"/>
+      <c r="G23" s="9" t="n">
         <v>-12000</v>
       </c>
-      <c r="H23" s="6" t="n"/>
-      <c r="I23" s="6" t="n"/>
-      <c r="J23" s="15">
+      <c r="H23" s="9" t="n"/>
+      <c r="I23" s="9" t="n"/>
+      <c r="J23" s="17">
         <f>SUM(D23:I23)</f>
         <v/>
       </c>
     </row>
     <row r="24">
-      <c r="B24" s="17" t="inlineStr">
+      <c r="B24" s="19" t="inlineStr">
         <is>
           <t xml:space="preserve">     (=) Lucro Bruto</t>
         </is>
       </c>
-      <c r="D24" s="18">
+      <c r="D24" s="20">
         <f>SUM(D22:D23)</f>
         <v/>
       </c>
-      <c r="E24" s="18">
+      <c r="E24" s="20">
         <f>SUM(E22:E23)</f>
         <v/>
       </c>
-      <c r="F24" s="18">
+      <c r="F24" s="20">
         <f>SUM(F22:F23)</f>
         <v/>
       </c>
-      <c r="G24" s="18">
+      <c r="G24" s="20">
         <f>SUM(G22:G23)</f>
         <v/>
       </c>
-      <c r="H24" s="18">
+      <c r="H24" s="20">
         <f>SUM(H22:H23)</f>
         <v/>
       </c>
-      <c r="I24" s="18">
+      <c r="I24" s="20">
         <f>SUM(I22:I23)</f>
         <v/>
       </c>
-      <c r="J24" s="18">
+      <c r="J24" s="20">
         <f>SUM(J22:J23)</f>
         <v/>
       </c>
@@ -2311,56 +2401,56 @@
           <t>(-) Despesas Operacionais</t>
         </is>
       </c>
-      <c r="D25" s="6" t="n"/>
-      <c r="E25" s="6" t="n"/>
-      <c r="F25" s="6" t="n"/>
-      <c r="G25" s="6" t="n"/>
-      <c r="H25" s="6" t="n">
+      <c r="D25" s="9" t="n"/>
+      <c r="E25" s="9" t="n"/>
+      <c r="F25" s="9" t="n"/>
+      <c r="G25" s="9" t="n"/>
+      <c r="H25" s="9" t="n">
         <v>-6000</v>
       </c>
-      <c r="I25" s="6" t="n"/>
-      <c r="J25" s="15">
+      <c r="I25" s="9" t="n"/>
+      <c r="J25" s="17">
         <f>SUM(D25:I25)</f>
         <v/>
       </c>
     </row>
     <row r="26">
-      <c r="B26" s="17" t="inlineStr">
+      <c r="B26" s="19" t="inlineStr">
         <is>
           <t xml:space="preserve">     (=) EBIT e Lucro Líquido</t>
         </is>
       </c>
-      <c r="D26" s="18">
+      <c r="D26" s="20">
         <f>SUM(D24:D25)</f>
         <v/>
       </c>
-      <c r="E26" s="18">
+      <c r="E26" s="20">
         <f>SUM(E24:E25)</f>
         <v/>
       </c>
-      <c r="F26" s="18">
+      <c r="F26" s="20">
         <f>SUM(F24:F25)</f>
         <v/>
       </c>
-      <c r="G26" s="18">
+      <c r="G26" s="20">
         <f>SUM(G24:G25)</f>
         <v/>
       </c>
-      <c r="H26" s="18">
+      <c r="H26" s="20">
         <f>SUM(H24:H25)</f>
         <v/>
       </c>
-      <c r="I26" s="18">
+      <c r="I26" s="20">
         <f>SUM(I24:I25)</f>
         <v/>
       </c>
-      <c r="J26" s="18">
+      <c r="J26" s="20">
         <f>SUM(J24:J25)</f>
         <v/>
       </c>
     </row>
     <row r="28">
-      <c r="B28" s="11" t="inlineStr">
+      <c r="B28" s="13" t="inlineStr">
         <is>
           <t>Demonstração dos Fluxos de Caixa</t>
         </is>
@@ -2383,43 +2473,43 @@
       <c r="I28" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="J28" s="11" t="inlineStr">
+      <c r="J28" s="13" t="inlineStr">
         <is>
           <t>Mês 1</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="B29" s="17" t="inlineStr">
+      <c r="B29" s="19" t="inlineStr">
         <is>
           <t>OPERAÇÕES</t>
         </is>
       </c>
-      <c r="D29" s="18">
+      <c r="D29" s="20">
         <f>SUM(D30:D32)</f>
         <v/>
       </c>
-      <c r="E29" s="18">
+      <c r="E29" s="20">
         <f>SUM(E30:E32)</f>
         <v/>
       </c>
-      <c r="F29" s="18">
+      <c r="F29" s="20">
         <f>SUM(F30:F32)</f>
         <v/>
       </c>
-      <c r="G29" s="18">
+      <c r="G29" s="20">
         <f>SUM(G30:G32)</f>
         <v/>
       </c>
-      <c r="H29" s="18">
+      <c r="H29" s="20">
         <f>SUM(H30:H32)</f>
         <v/>
       </c>
-      <c r="I29" s="18">
+      <c r="I29" s="20">
         <f>SUM(I30:I32)</f>
         <v/>
       </c>
-      <c r="J29" s="18">
+      <c r="J29" s="20">
         <f>SUM(J30:J32)</f>
         <v/>
       </c>
@@ -2430,15 +2520,15 @@
           <t>Recebimentos de Clientes</t>
         </is>
       </c>
-      <c r="D30" s="6" t="n"/>
-      <c r="E30" s="6" t="n"/>
-      <c r="F30" s="6" t="n"/>
-      <c r="G30" s="6" t="n">
+      <c r="D30" s="9" t="n"/>
+      <c r="E30" s="9" t="n"/>
+      <c r="F30" s="9" t="n"/>
+      <c r="G30" s="9" t="n">
         <v>27000</v>
       </c>
-      <c r="H30" s="6" t="n"/>
-      <c r="I30" s="6" t="n"/>
-      <c r="J30" s="15">
+      <c r="H30" s="9" t="n"/>
+      <c r="I30" s="9" t="n"/>
+      <c r="J30" s="17">
         <f>SUM(D30:I30)</f>
         <v/>
       </c>
@@ -2449,17 +2539,17 @@
           <t>Pagamentos a Fornecedores</t>
         </is>
       </c>
-      <c r="D31" s="6" t="n"/>
-      <c r="E31" s="6" t="n"/>
-      <c r="F31" s="6" t="n">
+      <c r="D31" s="9" t="n"/>
+      <c r="E31" s="9" t="n"/>
+      <c r="F31" s="9" t="n">
         <v>-12000</v>
       </c>
-      <c r="G31" s="6" t="n"/>
-      <c r="H31" s="6" t="n"/>
-      <c r="I31" s="6" t="n">
+      <c r="G31" s="9" t="n"/>
+      <c r="H31" s="9" t="n"/>
+      <c r="I31" s="9" t="n">
         <v>-6000</v>
       </c>
-      <c r="J31" s="15">
+      <c r="J31" s="17">
         <f>SUM(D31:I31)</f>
         <v/>
       </c>
@@ -2470,50 +2560,50 @@
           <t>Pagamentos de Despesas</t>
         </is>
       </c>
-      <c r="D32" s="6" t="n"/>
-      <c r="E32" s="6" t="n"/>
-      <c r="F32" s="6" t="n"/>
-      <c r="G32" s="6" t="n"/>
-      <c r="H32" s="6" t="n">
+      <c r="D32" s="9" t="n"/>
+      <c r="E32" s="9" t="n"/>
+      <c r="F32" s="9" t="n"/>
+      <c r="G32" s="9" t="n"/>
+      <c r="H32" s="9" t="n">
         <v>-6000</v>
       </c>
-      <c r="I32" s="6" t="n"/>
-      <c r="J32" s="15">
+      <c r="I32" s="9" t="n"/>
+      <c r="J32" s="17">
         <f>SUM(D32:I32)</f>
         <v/>
       </c>
     </row>
     <row r="33">
-      <c r="B33" s="17" t="inlineStr">
+      <c r="B33" s="19" t="inlineStr">
         <is>
           <t>INVESTIMENTOS</t>
         </is>
       </c>
-      <c r="D33" s="18">
+      <c r="D33" s="20">
         <f>SUM(D34:D34)</f>
         <v/>
       </c>
-      <c r="E33" s="18">
+      <c r="E33" s="20">
         <f>SUM(E34:E34)</f>
         <v/>
       </c>
-      <c r="F33" s="18">
+      <c r="F33" s="20">
         <f>SUM(F34:F34)</f>
         <v/>
       </c>
-      <c r="G33" s="18">
+      <c r="G33" s="20">
         <f>SUM(G34:G34)</f>
         <v/>
       </c>
-      <c r="H33" s="18">
+      <c r="H33" s="20">
         <f>SUM(H34:H34)</f>
         <v/>
       </c>
-      <c r="I33" s="18">
+      <c r="I33" s="20">
         <f>SUM(I34:I34)</f>
         <v/>
       </c>
-      <c r="J33" s="18">
+      <c r="J33" s="20">
         <f>SUM(J34:J34)</f>
         <v/>
       </c>
@@ -2524,50 +2614,50 @@
           <t>Aquisição de Imobilizado</t>
         </is>
       </c>
-      <c r="D34" s="6" t="n"/>
-      <c r="E34" s="6" t="n">
+      <c r="D34" s="9" t="n"/>
+      <c r="E34" s="9" t="n">
         <v>-30000</v>
       </c>
-      <c r="F34" s="6" t="n"/>
-      <c r="G34" s="6" t="n"/>
-      <c r="H34" s="6" t="n"/>
-      <c r="I34" s="6" t="n"/>
-      <c r="J34" s="15">
+      <c r="F34" s="9" t="n"/>
+      <c r="G34" s="9" t="n"/>
+      <c r="H34" s="9" t="n"/>
+      <c r="I34" s="9" t="n"/>
+      <c r="J34" s="17">
         <f>SUM(D34:I34)</f>
         <v/>
       </c>
     </row>
     <row r="35">
-      <c r="B35" s="17" t="inlineStr">
+      <c r="B35" s="19" t="inlineStr">
         <is>
           <t>FINANCIAMENTOS</t>
         </is>
       </c>
-      <c r="D35" s="18">
+      <c r="D35" s="20">
         <f>SUM(D36:D36)</f>
         <v/>
       </c>
-      <c r="E35" s="18">
+      <c r="E35" s="20">
         <f>SUM(E36:E36)</f>
         <v/>
       </c>
-      <c r="F35" s="18">
+      <c r="F35" s="20">
         <f>SUM(F36:F36)</f>
         <v/>
       </c>
-      <c r="G35" s="18">
+      <c r="G35" s="20">
         <f>SUM(G36:G36)</f>
         <v/>
       </c>
-      <c r="H35" s="18">
+      <c r="H35" s="20">
         <f>SUM(H36:H36)</f>
         <v/>
       </c>
-      <c r="I35" s="18">
+      <c r="I35" s="20">
         <f>SUM(I36:I36)</f>
         <v/>
       </c>
-      <c r="J35" s="18">
+      <c r="J35" s="20">
         <f>SUM(J36:J36)</f>
         <v/>
       </c>
@@ -2578,50 +2668,50 @@
           <t>Ingresso de Capital</t>
         </is>
       </c>
-      <c r="D36" s="6" t="n">
+      <c r="D36" s="9" t="n">
         <v>80000</v>
       </c>
-      <c r="E36" s="6" t="n"/>
-      <c r="F36" s="6" t="n"/>
-      <c r="G36" s="6" t="n"/>
-      <c r="H36" s="6" t="n"/>
-      <c r="I36" s="6" t="n"/>
-      <c r="J36" s="15">
+      <c r="E36" s="9" t="n"/>
+      <c r="F36" s="9" t="n"/>
+      <c r="G36" s="9" t="n"/>
+      <c r="H36" s="9" t="n"/>
+      <c r="I36" s="9" t="n"/>
+      <c r="J36" s="17">
         <f>SUM(D36:I36)</f>
         <v/>
       </c>
     </row>
     <row r="37">
-      <c r="B37" s="17" t="inlineStr">
+      <c r="B37" s="19" t="inlineStr">
         <is>
           <t>VARIAÇÃO NO CAIXA</t>
         </is>
       </c>
-      <c r="D37" s="18">
+      <c r="D37" s="20">
         <f>D29+D33+D35</f>
         <v/>
       </c>
-      <c r="E37" s="18">
+      <c r="E37" s="20">
         <f>E29+E33+E35</f>
         <v/>
       </c>
-      <c r="F37" s="18">
+      <c r="F37" s="20">
         <f>F29+F33+F35</f>
         <v/>
       </c>
-      <c r="G37" s="18">
+      <c r="G37" s="20">
         <f>G29+G33+G35</f>
         <v/>
       </c>
-      <c r="H37" s="18">
+      <c r="H37" s="20">
         <f>H29+H33+H35</f>
         <v/>
       </c>
-      <c r="I37" s="18">
+      <c r="I37" s="20">
         <f>I29+I33+I35</f>
         <v/>
       </c>
-      <c r="J37" s="18">
+      <c r="J37" s="20">
         <f>J29+J33+J35</f>
         <v/>
       </c>
@@ -2632,34 +2722,34 @@
           <t xml:space="preserve">    Saldo inicial de caixa</t>
         </is>
       </c>
-      <c r="J38" s="14" t="n">
+      <c r="J38" s="16" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="39">
-      <c r="B39" s="17" t="inlineStr">
+      <c r="B39" s="19" t="inlineStr">
         <is>
           <t xml:space="preserve">    Saldo final de caixa</t>
         </is>
       </c>
-      <c r="J39" s="15">
+      <c r="J39" s="17">
         <f>J38+J37</f>
         <v/>
       </c>
     </row>
     <row r="41">
-      <c r="B41" s="19" t="inlineStr">
+      <c r="B41" s="21" t="inlineStr">
         <is>
           <t>Caixa final da DFC menos Caixa do BP (tem que dar zero)</t>
         </is>
       </c>
-      <c r="J41" s="15">
+      <c r="J41" s="17">
         <f>J39-J6</f>
         <v/>
       </c>
     </row>
     <row r="43">
-      <c r="B43" s="11" t="inlineStr">
+      <c r="B43" s="13" t="inlineStr">
         <is>
           <t>Indicadores (automáticos)</t>
         </is>
@@ -2671,7 +2761,7 @@
           <t>Margem bruta</t>
         </is>
       </c>
-      <c r="J44" s="21">
+      <c r="J44" s="23">
         <f>IF(J22=0,"",J24/J22)</f>
         <v/>
       </c>
@@ -2682,7 +2772,7 @@
           <t>Margem líquida</t>
         </is>
       </c>
-      <c r="J45" s="21">
+      <c r="J45" s="23">
         <f>IF(J22=0,"",J26/J22)</f>
         <v/>
       </c>
@@ -2693,7 +2783,7 @@
           <t>% financiado por capital próprio (PL / Ativo)</t>
         </is>
       </c>
-      <c r="J46" s="21">
+      <c r="J46" s="23">
         <f>IF(J10=0,"",SUM(J15:J16)/J10)</f>
         <v/>
       </c>
@@ -2704,7 +2794,7 @@
           <t>ROE (LL / PL final)</t>
         </is>
       </c>
-      <c r="J47" s="21">
+      <c r="J47" s="23">
         <f>IF(SUM(J15:J16)=0,"",J26/SUM(J15:J16))</f>
         <v/>
       </c>
@@ -2720,17 +2810,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H16"/>
+  <dimension ref="A1:K17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="11" customWidth="1" min="1" max="1"/>
-    <col width="52" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="4" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
-    <col width="4" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="46" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="3" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="3" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="8" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2743,14 +2836,14 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Uma linha por movimento. Se a transação mexe em duas contas do mesmo lado (ex: sai caixa, entra estoque), usa as duas linhas.</t>
+          <t>Uma linha por movimento: escreve a conta e o valor, com sinal. Transação que mexe em três contas do mesmo lado usa as três linhas. A coluna Check acusa se aquela transação fechou.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Transação</t>
+          <t>Nº</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -2763,333 +2856,474 @@
           <t>ATIVO</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="4" t="n"/>
+      <c r="E4" s="3" t="inlineStr">
         <is>
           <t>=</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="F4" s="3" t="inlineStr">
         <is>
           <t>PASSIVO</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="G4" s="4" t="n"/>
+      <c r="H4" s="3" t="inlineStr">
         <is>
           <t>+</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="I4" s="3" t="inlineStr">
         <is>
           <t>PATRIMÔNIO LÍQUIDO</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr">
+      <c r="J4" s="4" t="n"/>
+      <c r="K4" s="3" t="inlineStr">
         <is>
           <t>Check</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="15" customHeight="1">
-      <c r="A5" s="4" t="n">
+    <row r="5">
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>conta</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>valor</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>conta</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>valor</t>
+        </is>
+      </c>
+      <c r="I5" s="5" t="inlineStr">
+        <is>
+          <t>conta</t>
+        </is>
+      </c>
+      <c r="J5" s="5" t="inlineStr">
+        <is>
+          <t>valor</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="B5" s="5" t="inlineStr">
+      <c r="B6" s="7" t="inlineStr">
         <is>
           <t>Integralização de capital de R$ 80.000 em dinheiro</t>
         </is>
       </c>
-      <c r="C5" s="6" t="n">
+      <c r="C6" s="8" t="inlineStr">
+        <is>
+          <t>Caixa</t>
+        </is>
+      </c>
+      <c r="D6" s="9" t="n">
         <v>80000</v>
       </c>
-      <c r="D5" s="7" t="inlineStr">
+      <c r="E6" s="10" t="inlineStr">
         <is>
           <t>=</t>
         </is>
       </c>
-      <c r="E5" s="6" t="n"/>
-      <c r="F5" s="7" t="inlineStr">
+      <c r="F6" s="8" t="n"/>
+      <c r="G6" s="9" t="n"/>
+      <c r="H6" s="10" t="inlineStr">
         <is>
           <t>+</t>
         </is>
       </c>
-      <c r="G5" s="6" t="n">
+      <c r="I6" s="8" t="inlineStr">
+        <is>
+          <t>Capital Social</t>
+        </is>
+      </c>
+      <c r="J6" s="9" t="n">
         <v>80000</v>
       </c>
-      <c r="H5" s="8">
-        <f>IF(COUNT(C5:C6,E5:E6,G5:G6)=0,"",IF(SUM(C5:C6)-SUM(E5:E6)-SUM(G5:G6)=0,"✔","✗"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="6">
-      <c r="C6" s="6" t="n"/>
-      <c r="D6" s="7" t="inlineStr">
+      <c r="K6" s="6">
+        <f>IF(COUNT(D6:D7,G6:G7,J6:J7)=0,"",IF(SUM(D6:D7)-SUM(G6:G7)-SUM(J6:J7)=0,"✔","✗"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="C7" s="8" t="n"/>
+      <c r="D7" s="9" t="n"/>
+      <c r="E7" s="10" t="inlineStr">
         <is>
           <t>=</t>
         </is>
       </c>
-      <c r="E6" s="6" t="n"/>
-      <c r="F6" s="7" t="inlineStr">
+      <c r="F7" s="8" t="n"/>
+      <c r="G7" s="9" t="n"/>
+      <c r="H7" s="10" t="inlineStr">
         <is>
           <t>+</t>
         </is>
       </c>
-      <c r="G6" s="6" t="n"/>
-    </row>
-    <row r="7" ht="15" customHeight="1">
-      <c r="A7" s="4" t="n">
+      <c r="I7" s="8" t="n"/>
+      <c r="J7" s="9" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="B7" s="5" t="inlineStr">
+      <c r="B8" s="7" t="inlineStr">
         <is>
           <t>Compra à vista de máquina de espresso e mobiliário por R$ 30.000</t>
         </is>
       </c>
-      <c r="C7" s="6" t="n">
+      <c r="C8" s="8" t="inlineStr">
+        <is>
+          <t>Caixa</t>
+        </is>
+      </c>
+      <c r="D8" s="9" t="n">
         <v>-30000</v>
       </c>
-      <c r="D7" s="7" t="inlineStr">
+      <c r="E8" s="10" t="inlineStr">
         <is>
           <t>=</t>
         </is>
       </c>
-      <c r="E7" s="6" t="n"/>
-      <c r="F7" s="7" t="inlineStr">
+      <c r="F8" s="8" t="n"/>
+      <c r="G8" s="9" t="n"/>
+      <c r="H8" s="10" t="inlineStr">
         <is>
           <t>+</t>
         </is>
       </c>
-      <c r="G7" s="6" t="n"/>
-      <c r="H7" s="8">
-        <f>IF(COUNT(C7:C8,E7:E8,G7:G8)=0,"",IF(SUM(C7:C8)-SUM(E7:E8)-SUM(G7:G8)=0,"✔","✗"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="8">
-      <c r="C8" s="6" t="n">
+      <c r="I8" s="8" t="n"/>
+      <c r="J8" s="9" t="n"/>
+      <c r="K8" s="6">
+        <f>IF(COUNT(D8:D9,G8:G9,J8:J9)=0,"",IF(SUM(D8:D9)-SUM(G8:G9)-SUM(J8:J9)=0,"✔","✗"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>Imobilizado</t>
+        </is>
+      </c>
+      <c r="D9" s="9" t="n">
         <v>30000</v>
       </c>
-      <c r="D8" s="7" t="inlineStr">
+      <c r="E9" s="10" t="inlineStr">
         <is>
           <t>=</t>
         </is>
       </c>
-      <c r="E8" s="6" t="n"/>
-      <c r="F8" s="7" t="inlineStr">
+      <c r="F9" s="8" t="n"/>
+      <c r="G9" s="9" t="n"/>
+      <c r="H9" s="10" t="inlineStr">
         <is>
           <t>+</t>
         </is>
       </c>
-      <c r="G8" s="6" t="n"/>
-    </row>
-    <row r="9" ht="15" customHeight="1">
-      <c r="A9" s="4" t="n">
+      <c r="I9" s="8" t="n"/>
+      <c r="J9" s="9" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="B9" s="5" t="inlineStr">
+      <c r="B10" s="7" t="inlineStr">
         <is>
           <t>Compra de café e insumos por R$ 24.000, metade à vista e metade a prazo</t>
         </is>
       </c>
-      <c r="C9" s="6" t="n">
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>Caixa</t>
+        </is>
+      </c>
+      <c r="D10" s="9" t="n">
         <v>-12000</v>
       </c>
-      <c r="D9" s="7" t="inlineStr">
+      <c r="E10" s="10" t="inlineStr">
         <is>
           <t>=</t>
         </is>
       </c>
-      <c r="E9" s="6" t="n">
+      <c r="F10" s="8" t="inlineStr">
+        <is>
+          <t>Contas a Pagar</t>
+        </is>
+      </c>
+      <c r="G10" s="9" t="n">
         <v>12000</v>
       </c>
-      <c r="F9" s="7" t="inlineStr">
+      <c r="H10" s="10" t="inlineStr">
         <is>
           <t>+</t>
         </is>
       </c>
-      <c r="G9" s="6" t="n"/>
-      <c r="H9" s="8">
-        <f>IF(COUNT(C9:C10,E9:E10,G9:G10)=0,"",IF(SUM(C9:C10)-SUM(E9:E10)-SUM(G9:G10)=0,"✔","✗"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="10">
-      <c r="C10" s="6" t="n">
+      <c r="I10" s="8" t="n"/>
+      <c r="J10" s="9" t="n"/>
+      <c r="K10" s="6">
+        <f>IF(COUNT(D10:D11,G10:G11,J10:J11)=0,"",IF(SUM(D10:D11)-SUM(G10:G11)-SUM(J10:J11)=0,"✔","✗"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>Estoque</t>
+        </is>
+      </c>
+      <c r="D11" s="9" t="n">
         <v>24000</v>
       </c>
-      <c r="D10" s="7" t="inlineStr">
+      <c r="E11" s="10" t="inlineStr">
         <is>
           <t>=</t>
         </is>
       </c>
-      <c r="E10" s="6" t="n"/>
-      <c r="F10" s="7" t="inlineStr">
+      <c r="F11" s="8" t="n"/>
+      <c r="G11" s="9" t="n"/>
+      <c r="H11" s="10" t="inlineStr">
         <is>
           <t>+</t>
         </is>
       </c>
-      <c r="G10" s="6" t="n"/>
-    </row>
-    <row r="11" ht="15" customHeight="1">
-      <c r="A11" s="4" t="n">
+      <c r="I11" s="8" t="n"/>
+      <c r="J11" s="9" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="B11" s="5" t="inlineStr">
+      <c r="B12" s="7" t="inlineStr">
         <is>
           <t>Venda de metade do estoque por R$ 27.000 à vista (custo de R$ 12.000)</t>
         </is>
       </c>
-      <c r="C11" s="6" t="n">
+      <c r="C12" s="8" t="inlineStr">
+        <is>
+          <t>Caixa</t>
+        </is>
+      </c>
+      <c r="D12" s="9" t="n">
         <v>27000</v>
       </c>
-      <c r="D11" s="7" t="inlineStr">
+      <c r="E12" s="10" t="inlineStr">
         <is>
           <t>=</t>
         </is>
       </c>
-      <c r="E11" s="6" t="n"/>
-      <c r="F11" s="7" t="inlineStr">
+      <c r="F12" s="8" t="n"/>
+      <c r="G12" s="9" t="n"/>
+      <c r="H12" s="10" t="inlineStr">
         <is>
           <t>+</t>
         </is>
       </c>
-      <c r="G11" s="6" t="n">
+      <c r="I12" s="8" t="inlineStr">
+        <is>
+          <t>Lucros Acumulados</t>
+        </is>
+      </c>
+      <c r="J12" s="9" t="n">
         <v>15000</v>
       </c>
-      <c r="H11" s="8">
-        <f>IF(COUNT(C11:C12,E11:E12,G11:G12)=0,"",IF(SUM(C11:C12)-SUM(E11:E12)-SUM(G11:G12)=0,"✔","✗"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="12">
-      <c r="C12" s="6" t="n">
+      <c r="K12" s="6">
+        <f>IF(COUNT(D12:D13,G12:G13,J12:J13)=0,"",IF(SUM(D12:D13)-SUM(G12:G13)-SUM(J12:J13)=0,"✔","✗"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>Estoque</t>
+        </is>
+      </c>
+      <c r="D13" s="9" t="n">
         <v>-12000</v>
       </c>
-      <c r="D12" s="7" t="inlineStr">
+      <c r="E13" s="10" t="inlineStr">
         <is>
           <t>=</t>
         </is>
       </c>
-      <c r="E12" s="6" t="n"/>
-      <c r="F12" s="7" t="inlineStr">
+      <c r="F13" s="8" t="n"/>
+      <c r="G13" s="9" t="n"/>
+      <c r="H13" s="10" t="inlineStr">
         <is>
           <t>+</t>
         </is>
       </c>
-      <c r="G12" s="6" t="n"/>
-    </row>
-    <row r="13" ht="15" customHeight="1">
-      <c r="A13" s="4" t="n">
+      <c r="I13" s="8" t="n"/>
+      <c r="J13" s="9" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="B13" s="5" t="inlineStr">
+      <c r="B14" s="7" t="inlineStr">
         <is>
           <t>Pagamento de salários e aluguel do mês, R$ 6.000 à vista</t>
         </is>
       </c>
-      <c r="C13" s="6" t="n">
+      <c r="C14" s="8" t="inlineStr">
+        <is>
+          <t>Caixa</t>
+        </is>
+      </c>
+      <c r="D14" s="9" t="n">
         <v>-6000</v>
       </c>
-      <c r="D13" s="7" t="inlineStr">
+      <c r="E14" s="10" t="inlineStr">
         <is>
           <t>=</t>
         </is>
       </c>
-      <c r="E13" s="6" t="n"/>
-      <c r="F13" s="7" t="inlineStr">
+      <c r="F14" s="8" t="n"/>
+      <c r="G14" s="9" t="n"/>
+      <c r="H14" s="10" t="inlineStr">
         <is>
           <t>+</t>
         </is>
       </c>
-      <c r="G13" s="6" t="n">
+      <c r="I14" s="8" t="inlineStr">
+        <is>
+          <t>Lucros Acumulados</t>
+        </is>
+      </c>
+      <c r="J14" s="9" t="n">
         <v>-6000</v>
       </c>
-      <c r="H13" s="8">
-        <f>IF(COUNT(C13:C14,E13:E14,G13:G14)=0,"",IF(SUM(C13:C14)-SUM(E13:E14)-SUM(G13:G14)=0,"✔","✗"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="14">
-      <c r="C14" s="6" t="n"/>
-      <c r="D14" s="7" t="inlineStr">
+      <c r="K14" s="6">
+        <f>IF(COUNT(D14:D15,G14:G15,J14:J15)=0,"",IF(SUM(D14:D15)-SUM(G14:G15)-SUM(J14:J15)=0,"✔","✗"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="C15" s="8" t="n"/>
+      <c r="D15" s="9" t="n"/>
+      <c r="E15" s="10" t="inlineStr">
         <is>
           <t>=</t>
         </is>
       </c>
-      <c r="E14" s="6" t="n"/>
-      <c r="F14" s="7" t="inlineStr">
+      <c r="F15" s="8" t="n"/>
+      <c r="G15" s="9" t="n"/>
+      <c r="H15" s="10" t="inlineStr">
         <is>
           <t>+</t>
         </is>
       </c>
-      <c r="G14" s="6" t="n"/>
-    </row>
-    <row r="15" ht="15" customHeight="1">
-      <c r="A15" s="4" t="n">
+      <c r="I15" s="8" t="n"/>
+      <c r="J15" s="9" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="B15" s="5" t="inlineStr">
+      <c r="B16" s="7" t="inlineStr">
         <is>
           <t>Pagamento de metade do que devia aos fornecedores</t>
         </is>
       </c>
-      <c r="C15" s="6" t="n">
+      <c r="C16" s="8" t="inlineStr">
+        <is>
+          <t>Caixa</t>
+        </is>
+      </c>
+      <c r="D16" s="9" t="n">
         <v>-6000</v>
       </c>
-      <c r="D15" s="7" t="inlineStr">
+      <c r="E16" s="10" t="inlineStr">
         <is>
           <t>=</t>
         </is>
       </c>
-      <c r="E15" s="6" t="n">
+      <c r="F16" s="8" t="inlineStr">
+        <is>
+          <t>Contas a Pagar</t>
+        </is>
+      </c>
+      <c r="G16" s="9" t="n">
         <v>-6000</v>
       </c>
-      <c r="F15" s="7" t="inlineStr">
+      <c r="H16" s="10" t="inlineStr">
         <is>
           <t>+</t>
         </is>
       </c>
-      <c r="G15" s="6" t="n"/>
-      <c r="H15" s="8">
-        <f>IF(COUNT(C15:C16,E15:E16,G15:G16)=0,"",IF(SUM(C15:C16)-SUM(E15:E16)-SUM(G15:G16)=0,"✔","✗"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="16">
-      <c r="C16" s="6" t="n"/>
-      <c r="D16" s="7" t="inlineStr">
+      <c r="I16" s="8" t="n"/>
+      <c r="J16" s="9" t="n"/>
+      <c r="K16" s="6">
+        <f>IF(COUNT(D16:D17,G16:G17,J16:J17)=0,"",IF(SUM(D16:D17)-SUM(G16:G17)-SUM(J16:J17)=0,"✔","✗"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="C17" s="8" t="n"/>
+      <c r="D17" s="9" t="n"/>
+      <c r="E17" s="10" t="inlineStr">
         <is>
           <t>=</t>
         </is>
       </c>
-      <c r="E16" s="6" t="n"/>
-      <c r="F16" s="7" t="inlineStr">
+      <c r="F17" s="8" t="n"/>
+      <c r="G17" s="9" t="n"/>
+      <c r="H17" s="10" t="inlineStr">
         <is>
           <t>+</t>
         </is>
       </c>
-      <c r="G16" s="6" t="n"/>
+      <c r="I17" s="8" t="n"/>
+      <c r="J17" s="9" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="18">
-    <mergeCell ref="A5:A6"/>
-    <mergeCell ref="B9:B10"/>
-    <mergeCell ref="H5:H6"/>
-    <mergeCell ref="H13:H14"/>
-    <mergeCell ref="H9:H10"/>
-    <mergeCell ref="A9:A10"/>
-    <mergeCell ref="A13:A14"/>
-    <mergeCell ref="B13:B14"/>
-    <mergeCell ref="A15:A16"/>
-    <mergeCell ref="A7:A8"/>
-    <mergeCell ref="B7:B8"/>
-    <mergeCell ref="B11:B12"/>
-    <mergeCell ref="H7:H8"/>
-    <mergeCell ref="H15:H16"/>
-    <mergeCell ref="H11:H12"/>
-    <mergeCell ref="B5:B6"/>
-    <mergeCell ref="A11:A12"/>
-    <mergeCell ref="B15:B16"/>
+  <mergeCells count="21">
+    <mergeCell ref="F4:G4"/>
+    <mergeCell ref="B12:B13"/>
+    <mergeCell ref="B8:B9"/>
+    <mergeCell ref="A16:A17"/>
+    <mergeCell ref="A6:A7"/>
+    <mergeCell ref="B14:B15"/>
+    <mergeCell ref="C4:D4"/>
+    <mergeCell ref="A12:A13"/>
+    <mergeCell ref="K12:K13"/>
+    <mergeCell ref="B10:B11"/>
+    <mergeCell ref="B6:B7"/>
+    <mergeCell ref="A14:A15"/>
+    <mergeCell ref="A8:A9"/>
+    <mergeCell ref="K14:K15"/>
+    <mergeCell ref="K8:K9"/>
+    <mergeCell ref="A10:A11"/>
+    <mergeCell ref="K10:K11"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="K16:K17"/>
+    <mergeCell ref="K6:K7"/>
+    <mergeCell ref="B16:B17"/>
   </mergeCells>
+  <dataValidations count="3">
+    <dataValidation sqref="C6 C7 C8 C9 C10 C11 C12 C13 C14 C15 C16 C17" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Caixa,Estoque,Imobilizado"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F6 F7 F8 F9 F10 F11 F12 F13 F14 F15 F16 F17" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Contas a Pagar"</formula1>
+    </dataValidation>
+    <dataValidation sqref="I6 I7 I8 I9 I10 I11 I12 I13 I14 I15 I16 I17" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Capital Social,Lucros Acumulados"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
vault backup: 2026-08-10 19:18:15
</commit_message>
<xml_diff>
--- a/ContabilidadeFinanceira/Treinos/Ex1_GraoDeOuro.xlsx
+++ b/ContabilidadeFinanceira/Treinos/Ex1_GraoDeOuro.xlsx
@@ -920,7 +920,7 @@
       <c r="J17" s="9" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="21">
+  <mergeCells count="22">
     <mergeCell ref="F4:G4"/>
     <mergeCell ref="B12:B13"/>
     <mergeCell ref="B8:B9"/>
@@ -933,6 +933,7 @@
     <mergeCell ref="B10:B11"/>
     <mergeCell ref="B6:B7"/>
     <mergeCell ref="A14:A15"/>
+    <mergeCell ref="A1:D1"/>
     <mergeCell ref="A8:A9"/>
     <mergeCell ref="K14:K15"/>
     <mergeCell ref="K8:K9"/>
@@ -984,7 +985,7 @@
     <row r="1">
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Cafeteria Grão de Ouro  |  Mês 1  |  valores em R$</t>
+          <t>Cafeteria Grão de Ouro</t>
         </is>
       </c>
       <c r="D1" s="11" t="inlineStr">
@@ -994,6 +995,11 @@
       </c>
     </row>
     <row r="2" ht="42" customHeight="1">
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Mês 1  |  valores em R$</t>
+        </is>
+      </c>
       <c r="D2" s="12" t="inlineStr">
         <is>
           <t>Integralização de capital de R$ 80.000 em dinheiro</t>
@@ -1886,6 +1892,9 @@
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B1:C1"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1916,7 +1925,7 @@
     <row r="1">
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Cafeteria Grão de Ouro  |  Mês 1  |  valores em R$</t>
+          <t>Cafeteria Grão de Ouro</t>
         </is>
       </c>
       <c r="D1" s="11" t="inlineStr">
@@ -1926,6 +1935,11 @@
       </c>
     </row>
     <row r="2" ht="42" customHeight="1">
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Mês 1  |  valores em R$</t>
+        </is>
+      </c>
       <c r="D2" s="12" t="inlineStr">
         <is>
           <t>Integralização de capital de R$ 80.000 em dinheiro</t>
@@ -2800,6 +2814,9 @@
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B1:C1"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3290,7 +3307,7 @@
       <c r="J17" s="9" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="21">
+  <mergeCells count="22">
     <mergeCell ref="F4:G4"/>
     <mergeCell ref="B12:B13"/>
     <mergeCell ref="B8:B9"/>
@@ -3303,6 +3320,7 @@
     <mergeCell ref="B10:B11"/>
     <mergeCell ref="B6:B7"/>
     <mergeCell ref="A14:A15"/>
+    <mergeCell ref="A1:D1"/>
     <mergeCell ref="A8:A9"/>
     <mergeCell ref="K14:K15"/>
     <mergeCell ref="K8:K9"/>

</xml_diff>